<commit_message>
Mark rows as viewed on Next/Previous; resume at last viewed; show chunk row range 51-100; 100-word names in sample; e2e fixes
</commit_message>
<xml_diff>
--- a/samples/sample.xlsx
+++ b/samples/sample.xlsx
@@ -31,7 +31,28 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Person 1</t>
+    <t>finally your mostly more many without while old would its our get however would suddenly gradually eventually have gradually the through everyone she some its eventually quickly way them while obviously our that these sometimes will that had them its said put totally are especially but first will totally completely had without other gradually eventually always mostly your slowly new should they completely completely out where carefully than normally which this while with where man which you out someone recently without into about there mostly slowly finally let everything eventually use she mainly then with first from see primarily recently</t>
+  </si>
+  <si>
+    <t>Support</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>many not one therefore her put absolutely get there usually had because the your mostly boy everything its nothing fully obviously initially many should apparently that did before then was than its would quickly gradually before originally normally certainly after generally when many before her fully its perhaps gradually absolutely therefore each use when there her our quickly each completely definitely who anything been out more perhaps see our him then was apparently now particularly during although another can where exactly before recently they before one completely these during old normally completely but sometimes for was then each really will</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>always use how boy generally his one all basically during these that for primarily definitely these its who carefully only immediately and nothing someone there totally into definitely that about between too man particularly been mainly one should she put before this his without then way only but use first particularly completely would absolutely during was many everything definitely see your put exactly partly being before the partly carefully out them initially another apparently say not everyone first our say she where way there being generally before because them immediately slowly new after had everything absolutely certainly one man old</t>
   </si>
   <si>
     <t>Finance</t>
@@ -40,568 +61,547 @@
     <t>Rejected</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Person 2</t>
-  </si>
-  <si>
-    <t>Support</t>
-  </si>
-  <si>
-    <t>Approved</t>
-  </si>
-  <si>
-    <t>Person 3</t>
+    <t>but entirely although you nothing another eventually usually although into although are and everyone although old when therefore use each slowly absolutely should perhaps everyone anything boy now this slowly could many recently now new when another entirely where completely there quickly could other she someone all but between originally absolutely mainly while slowly their gradually who was mainly their originally you which usually your has slowly you everything slowly put boy all between without therefore they while with partly obviously other mainly would many generally through say now into suddenly for while that their first use really perhaps has</t>
   </si>
   <si>
     <t>Sales</t>
   </si>
   <si>
-    <t>Person 4</t>
-  </si>
-  <si>
-    <t>Person 5</t>
-  </si>
-  <si>
-    <t>Pending</t>
+    <t>some anything usually all when would because obviously totally generally old all quickly way initially you after quickly which more way basically absolutely many during into after usually that however anything particularly apparently while some actually between will especially obviously certainly with that had you initially now already are into old primarily more have from him partly new each where out before out out day while put was will our who are gradually way during basically would more should which eventually his other out everyone say new through without these that because her immediately nothing between carefully where generally normally</t>
   </si>
   <si>
     <t>Note for row 5</t>
   </si>
   <si>
-    <t>Person 6</t>
+    <t>and immediately first put will where first about immediately some our him through everyone recently did before this how are exactly really through then immediately him should usually through sometimes sometimes has been therefore initially day completely many use one say too not normally slowly they sometimes certainly absolutely apparently put carefully originally apparently suddenly totally but all exactly each mainly something however are let however said everyone recently more now would would use our their anything everything mostly way new after always did our anything someone get fully perhaps would obviously actually let when than always our him eventually</t>
+  </si>
+  <si>
+    <t>Engineering</t>
+  </si>
+  <si>
+    <t>Needs Review</t>
+  </si>
+  <si>
+    <t>did boy finally immediately slowly immediately quickly way see therefore its with certainly which old actually immediately something carefully not finally normally old totally that all has recently been put other normally only let boy only quickly see but the from and how mostly day primarily sometimes which another see their been but mainly usually for perhaps each usually them they did him basically him them another definitely its fully not being another between should especially would although when originally there primarily use you other boy see new who another which said entirely during her their where could there the</t>
+  </si>
+  <si>
+    <t>another because completely immediately them that about boy many normally mostly day certainly you all day have his but nothing now new always have who eventually said they something immediately recently someone than into immediately did say one therefore the totally him new eventually and from primarily should other out anything before sometimes initially boy basically another another each been generally mainly apparently from mostly from each each recently him completely because generally basically and where during slowly absolutely too fully with generally everyone new actually get said out how recently how which was through before them basically entirely perhaps</t>
+  </si>
+  <si>
+    <t>how has have slowly him all would basically new should the immediately sometimes immediately sometimes therefore being quickly the really originally old without between get completely without everything had however has they your recently her when their basically anything get slowly all certainly already too entirely who slowly how these them him entirely now everyone certainly she its how this immediately but these normally where has has her partly are actually did through said see absolutely say especially can recently about exactly quickly into the exactly all get completely without definitely primarily should basically that gradually finally anything she apparently</t>
   </si>
   <si>
     <t>In Progress</t>
   </si>
   <si>
-    <t>Person 7</t>
-  </si>
-  <si>
-    <t>Person 8</t>
+    <t>particularly only you through some put this immediately our see now before how new from now absolutely than suddenly exactly after quickly been its nothing when mostly while not therefore between already suddenly carefully some many use had have however from fully suddenly where recently originally mostly fully exactly been will can how said not sometimes should partly with which for said finally eventually our did recently how our she immediately after although say normally our will too she because slowly always initially eventually man quickly while without said normally mostly will sometimes your particularly primarily into during immediately who</t>
+  </si>
+  <si>
+    <t>Note for row 10</t>
+  </si>
+  <si>
+    <t>fully him apparently normally many who other there usually fully his use out someone have other where after where day anything only put initially use other perhaps and been should always absolutely day gradually suddenly especially immediately although slowly let suddenly mainly this now boy each not into other certainly they are him their way perhaps for are its originally more suddenly did our been basically our originally out being some that but let certainly already particularly day normally actually anything are him completely entirely totally use after first was did way said absolutely generally slowly there originally actually see</t>
+  </si>
+  <si>
+    <t>but their put that everyone slowly for only obviously someone carefully not then new get you being one said the quickly especially old our originally from suddenly recently for many normally immediately has they new always they basically slowly should recently can would definitely mostly although mostly however another boy perhaps this during without will have obviously finally another finally been man man always everyone everything normally did let therefore your one old you her did while but these him the where there from then will who how are particularly the had get everyone everything absolutely man are are not</t>
+  </si>
+  <si>
+    <t>did quickly anything which through completely and use all obviously but carefully totally her basically she one way suddenly way him apparently how being recently eventually not slowly actually our who not when carefully old fully usually slowly have way and fully being but then fully basically being entirely some one after however with now boy where that with especially nothing everything primarily really eventually absolutely obviously absolutely quickly primarily gradually for they another been fully apparently completely certainly they many while perhaps suddenly only are your eventually man basically they for how should usually into was basically said someone</t>
+  </si>
+  <si>
+    <t>slowly them through not mainly these totally really especially our how old always apparently immediately absolutely out his than everything exactly then man sometimes anything man totally did suddenly all will although because nothing did partly their quickly would everything from man did which something all although said its have obviously was originally will always some someone day new said perhaps with him let can while sometimes say boy primarily entirely when everything but recently apparently actually something suddenly the especially suddenly him how perhaps but normally each already out only the the actually where her everything another mainly their</t>
+  </si>
+  <si>
+    <t>this only initially she through had fully boy generally basically carefully already was their said which then everything them perhaps out from eventually someone without slowly generally the for but slowly the particularly put sometimes his could really boy mostly sometimes quickly slowly everyone gradually fully always was was let not primarily other their someone then and although after first between when some him another everything immediately totally old perhaps nothing mostly immediately absolutely mainly than said for generally have someone has old see already exactly one his you get say would absolutely they there immediately old these absolutely particularly</t>
+  </si>
+  <si>
+    <t>Note for row 15</t>
+  </si>
+  <si>
+    <t>all gradually day immediately our really their your has definitely however which too immediately carefully fully perhaps this initially how too between someone use carefully slowly everyone normally these where but certainly than her put while who however who each actually and day being his before already someone there use slowly actually all how not particularly old let primarily him can one all obviously more his there already absolutely our say too out totally fully its although always say been she through someone while our too being after them already gradually now them primarily finally man old which first you</t>
+  </si>
+  <si>
+    <t>between immediately get anything suddenly during immediately entirely let generally immediately originally immediately now the between suddenly however finally mainly everything new get how see man let really could into immediately when man totally other her immediately exactly immediately initially had too perhaps being carefully something from our too for than because put finally completely anything our they sometimes said out something how definitely this sometimes from can anything about boy she another during not use before gradually anything many entirely she immediately into there before nothing your quickly this use exactly mostly normally after someone because let can but</t>
+  </si>
+  <si>
+    <t>totally should other for quickly carefully another now them her into her someone therefore suddenly obviously immediately her old then new that obviously old mainly everything being between other sometimes too perhaps another primarily can can who generally being these for will her some basically how perhaps can then suddenly for other generally way mostly was everything mainly put gradually suddenly her now mainly suddenly how initially exactly there than however especially although eventually first how sometimes not how really each way how did old for which let without without suddenly after all gradually more all that after are totally</t>
+  </si>
+  <si>
+    <t>completely use will about other than these anything who should day mainly way new this put use certainly but exactly especially partly therefore could everyone all through suddenly say although when who however the say about everyone finally therefore already originally had someone can all when our our they while other another eventually suddenly and first recently although then him mainly everything only all his before these one immediately about then actually she during this other primarily old nothing where their mostly and first however into who old obviously really should now while someone before where are than exactly really</t>
+  </si>
+  <si>
+    <t>definitely because suddenly has being was new the his which while immediately fully but especially basically particularly more other certainly sometimes from see because into say out first them all during did they especially then him her our who day day eventually suddenly out boy exactly especially them especially each another can perhaps boy the you someone would mostly basically let who how each suddenly your have there another these could where all they had another should because anything and although therefore which how already and without about exactly who apparently before say gradually nothing carefully man all carefully however</t>
+  </si>
+  <si>
+    <t>Note for row 20</t>
+  </si>
+  <si>
+    <t>his basically been basically however way quickly their many where for because everything first too slowly however particularly everyone nothing first new will therefore her being one too them from someone certainly these through perhaps you man now definitely immediately totally its how which immediately let finally exactly her now through him but during being can partly exactly gradually where about your for where really this partly only which you usually our many certainly these each get old during her sometimes entirely after see our the while say get use through said the some not has without first but say</t>
+  </si>
+  <si>
+    <t>who gradually because for because say entirely about while perhaps you more without entirely our into you where then but had without totally have all will mostly then have because perhaps after your because after totally immediately have sometimes before certainly perhaps his however there everyone immediately normally this day from suddenly who they has generally recently his before had boy that then basically too she had really their your between mostly let obviously this first about normally absolutely said but their carefully old particularly say finally only where another before let entirely especially this everything everyone see their than</t>
+  </si>
+  <si>
+    <t>was being too into usually recently their apparently boy definitely mostly exactly eventually exactly how first should other about while and because did how into her your originally did not our could apparently although always although many someone completely therefore can usually through with another carefully finally being basically anything slowly will normally already their him after mostly but and could they its said finally immediately its totally only basically when initially being should say without the let something boy new always than primarily them for there particularly your exactly absolutely has this first its only already eventually between sometimes</t>
+  </si>
+  <si>
+    <t>however way let for was primarily already now not him the these initially there too are recently has gradually should completely all after basically did about always certainly finally and particularly other more however could something all for will between into however someone out say but obviously then during generally and because have get someone than originally carefully these many who another let boy finally now into however let through old now usually especially finally get with than will someone but many definitely everything has particularly can boy was obviously after are him has already certainly mostly more the always</t>
   </si>
   <si>
     <t>HR</t>
   </si>
   <si>
-    <t>Person 9</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>Person 10</t>
-  </si>
-  <si>
-    <t>Note for row 10</t>
-  </si>
-  <si>
-    <t>Person 11</t>
-  </si>
-  <si>
-    <t>Person 12</t>
-  </si>
-  <si>
-    <t>Person 13</t>
-  </si>
-  <si>
-    <t>Person 14</t>
-  </si>
-  <si>
-    <t>Needs Review</t>
-  </si>
-  <si>
-    <t>Person 15</t>
-  </si>
-  <si>
-    <t>Engineering</t>
-  </si>
-  <si>
-    <t>Note for row 15</t>
-  </si>
-  <si>
-    <t>Person 16</t>
-  </si>
-  <si>
-    <t>Person 17</t>
-  </si>
-  <si>
-    <t>Person 18</t>
-  </si>
-  <si>
-    <t>Person 19</t>
-  </si>
-  <si>
-    <t>Person 20</t>
-  </si>
-  <si>
-    <t>Note for row 20</t>
-  </si>
-  <si>
-    <t>Person 21</t>
-  </si>
-  <si>
-    <t>Person 22</t>
-  </si>
-  <si>
-    <t>Person 23</t>
-  </si>
-  <si>
-    <t>Person 24</t>
-  </si>
-  <si>
-    <t>Person 25</t>
+    <t>obviously has them which certainly only originally boy definitely usually particularly each quickly therefore partly have usually only use some already because more about all and which with nothing immediately has generally say initially one could there her will with therefore can certainly where and recently eventually this anything another boy actually new out because primarily with him quickly through eventually but use too all who therefore now old all anything after already when another now been into our perhaps from only after for its recently old everyone fully the some anything during only man did recently other you mostly</t>
   </si>
   <si>
     <t>Note for row 25</t>
   </si>
   <si>
-    <t>Person 26</t>
-  </si>
-  <si>
-    <t>Person 27</t>
-  </si>
-  <si>
-    <t>Person 28</t>
-  </si>
-  <si>
-    <t>Person 29</t>
-  </si>
-  <si>
-    <t>Person 30</t>
+    <t>basically obviously this definitely suddenly them use the than suddenly day suddenly let which are before mostly particularly old that has out that was will quickly originally did where have generally this that definitely actually there slowly for and not however our which too immediately are old let how some said mostly between old into after apparently man now suddenly new all into there say generally who being especially other can which totally only apparently completely into because another after everyone one how initially through finally basically particularly she see because for than mostly was many gradually certainly through certainly</t>
+  </si>
+  <si>
+    <t>because has your have our did totally quickly through totally then use our quickly quickly his from absolutely through see are the your finally there partly obviously someone therefore fully carefully which see certainly can more basically them new only partly put has gradually however however slowly old their did did boy primarily their him some when fully his see your during during boy more originally see between before when immediately everything while another nothing which anything they perhaps perhaps this with these not see after you your immediately day more can something through will totally this sometimes should being</t>
+  </si>
+  <si>
+    <t>who because especially him generally recently because partly always exactly only mostly without them between fully between everything who slowly man was more therefore already man way put are should already this through these can other than how was partly day and eventually then are how however sometimes entirely say when first exactly perhaps will between completely finally her from how mainly apparently been finally always for primarily apparently primarily certainly recently new nothing when only will without something day primarily all many put boy now use this boy eventually had the said get first fully for boy totally the</t>
+  </si>
+  <si>
+    <t>carefully boy basically absolutely originally because not immediately she nothing new everything should therefore but about when recently now them initially only for could someone without has there one not you fully before day has his quickly after not now but really completely however way could nothing then into entirely especially get out him his see where and being one way and apparently not how with exactly suddenly too will which new have which between she quickly had too with already all being after finally certainly something although did see where during quickly being originally initially generally let are while</t>
+  </si>
+  <si>
+    <t>one another therefore this that obviously completely its each generally way use and during through for always therefore said fully the immediately our they all immediately anything them new too during from have then our boy therefore who now now day slowly totally the totally while old being generally she which him before from therefore nothing something too when while something although can therefore they basically has originally another someone entirely because through everyone only suddenly there quickly before everyone gradually immediately recently said had see fully get the because many recently see everything them definitely for now only said</t>
   </si>
   <si>
     <t>Note for row 30</t>
   </si>
   <si>
-    <t>Person 31</t>
-  </si>
-  <si>
-    <t>Person 32</t>
-  </si>
-  <si>
-    <t>Person 33</t>
-  </si>
-  <si>
-    <t>Person 34</t>
-  </si>
-  <si>
-    <t>Person 35</t>
+    <t>therefore basically than now from them partly already there you gradually totally without more was actually see his primarily carefully one that first primarily has the man primarily from already everything get see then usually our generally during nothing her mainly our said some way for when way immediately said been she before your apparently partly would gradually your already mainly other this however normally entirely before apparently quickly immediately slowly can only one all are during them and entirely everything get mainly you way the should initially been partly was where slowly anything man many could than old new</t>
+  </si>
+  <si>
+    <t>really some with from everyone gradually when did generally carefully already she too other through fully another not into will mainly its perhaps everyone this another its you but normally there generally was immediately however many put get especially these during nothing old was for that fully would her man for really between way between before then with should because has definitely mainly after that was some apparently way first first completely nothing obviously him really you gradually you one let immediately who way which first partly therefore get put eventually boy use carefully gradually than out from before too</t>
+  </si>
+  <si>
+    <t>immediately use without that therefore because their them the been between nothing and being them basically their these with partly but new that always everything day through could through primarily now absolutely her perhaps out use while other new without its would originally everyone day some something eventually for before put generally between while there these everyone exactly who new the way his quickly between generally exactly during about some old partly really its slowly where other our let when only this was their then this more mainly more them use slowly immediately quickly let how suddenly these where there</t>
+  </si>
+  <si>
+    <t>see man obviously how gradually who immediately without now everyone basically quickly something immediately use definitely some another who recently could into their for suddenly usually its everyone been certainly and originally the absolutely suddenly will mainly certainly everything these more mainly who because not about had been because say let obviously man absolutely when about said had obviously and will these out could more man because her absolutely how immediately the there particularly would been immediately completely however partly eventually she gradually old but too let before for some are something finally boy really said particularly for from really</t>
+  </si>
+  <si>
+    <t>completely everyone sometimes because first new boy obviously apparently can old first perhaps did always everyone where its totally immediately anything she way only with apparently when who these always everyone anything its apparently actually about totally each perhaps not his their its absolutely your another day partly into and without something put while that between more she suddenly many way apparently say should more how old although have something more originally about apparently them after not can during initially while other many suddenly anything normally exactly way these definitely where these absolutely already usually way who carefully during more</t>
   </si>
   <si>
     <t>Note for row 35</t>
   </si>
   <si>
-    <t>Person 36</t>
-  </si>
-  <si>
-    <t>Person 37</t>
-  </si>
-  <si>
-    <t>Person 38</t>
-  </si>
-  <si>
-    <t>Person 39</t>
-  </si>
-  <si>
-    <t>Person 40</t>
+    <t>generally than slowly the definitely when fully before mostly for the can while did that perhaps been put always especially obviously one have completely his said not eventually entirely gradually totally some therefore already would completely with gradually from which suddenly where you partly these out however first say finally could fully initially immediately especially everyone put first however eventually originally already this someone did usually let definitely obviously boy where where already her finally from before slowly this then way their they obviously will they some than how would about partly into say how some than obviously eventually man</t>
+  </si>
+  <si>
+    <t>really put them certainly have these but exactly each each certainly another these apparently although primarily been let him more being while been because usually old obviously where mainly too where she who has initially initially man your slowly his how into apparently quickly way finally get they being always your day initially some someone where usually about see after use perhaps not than which could him really how however had without nothing carefully nothing partly but with she immediately out all basically they another them really obviously before always let eventually always sometimes suddenly other was quickly certainly more</t>
+  </si>
+  <si>
+    <t>one sometimes apparently had before basically let usually said said therefore normally than day actually someone everyone other while someone could only our our without have definitely already been has see been recently from sometimes will has its other primarily there would say his definitely them completely first someone some initially not slowly could boy while usually and especially through suddenly totally fully before our when usually generally exactly because primarily normally actually how been boy would immediately see you carefully nothing would there said about then sometimes perhaps everyone another her there new many day after them someone its</t>
+  </si>
+  <si>
+    <t>always before exactly sometimes everyone this how him completely therefore will would many obviously completely without although each finally said did only its too them between the another sometimes primarily someone finally the nothing absolutely there totally her initially these this put other new now before mainly who will out there boy for for you they this without all gradually get its that without originally normally some man originally let than between generally her than the already therefore which boy nothing sometimes one has now that said something they nothing normally each than see its primarily said obviously then being</t>
+  </si>
+  <si>
+    <t>than old the completely where their particularly than you totally which can absolutely first could actually originally something about about other immediately see new everything will all finally all slowly particularly could certainly put completely had has quickly said let been immediately actually say recently which can them without mostly see can particularly and did the between where certainly where this him them definitely into absolutely with always recently who finally boy our however obviously anything absolutely get immediately have put with however she perhaps through that without has exactly carefully carefully she primarily did into see between because into</t>
   </si>
   <si>
     <t>Note for row 40</t>
   </si>
   <si>
-    <t>Person 41</t>
-  </si>
-  <si>
-    <t>Person 42</t>
-  </si>
-  <si>
-    <t>Person 43</t>
-  </si>
-  <si>
-    <t>Person 44</t>
-  </si>
-  <si>
-    <t>Person 45</t>
+    <t>have her without nothing only therefore immediately everyone have generally out suddenly she sometimes this certainly another sometimes exactly how with where without particularly completely many you exactly her they everything nothing each for completely can out many immediately put obviously generally old has slowly you too was too some someone completely could perhaps mainly say all really always you has something gradually too basically you after use put suddenly each immediately already and apparently immediately many its from another day suddenly through she put and first them quickly immediately his actually into use that quickly completely particularly these before</t>
+  </si>
+  <si>
+    <t>therefore out carefully are did because partly old originally nothing normally because only because him out originally everything she more everyone exactly some all will put into the apparently everything then their without suddenly nothing there man get obviously put use where did everything especially already without anything who out slowly would although therefore about new for some will while immediately definitely quickly immediately should completely generally however had something finally but way without entirely her after you through perhaps really now too recently our new basically particularly another its boy its mainly quickly quickly see this really completely between</t>
+  </si>
+  <si>
+    <t>one did between our carefully use now nothing only have let mostly she slowly initially their nothing had first but should about would many him initially other put which absolutely then you especially generally old use with therefore finally would normally after therefore you carefully really where then normally quickly our her its with your suddenly way originally being about should generally after with after already more someone everything during recently day absolutely usually him now generally say man finally before particularly basically then her another fully into put all normally originally before into already usually there being these but</t>
+  </si>
+  <si>
+    <t>only entirely but how their nothing said this immediately man has certainly their perhaps mainly everything they mainly its because actually certainly usually which have too only partly during had everyone because that did was mostly during your before too after would see basically this into not where too you always although use normally primarily did the being especially completely with they its not put they now him therefore should can did sometimes not some particularly apparently should gradually without your finally only get should some and not this these will nothing that been will however said its all way</t>
+  </si>
+  <si>
+    <t>some another out they definitely one obviously about how finally quickly now had new where see new let mostly will eventually was some gradually about everything that therefore boy these nothing perhaps with although where entirely being recently after they was everyone immediately not really said absolutely some that recently everything certainly eventually did they totally anything the will you how will put recently everything usually partly many your get the will therefore usually fully boy although can from however obviously initially day would there really someone can however generally before certainly where have new mainly could will someone would</t>
   </si>
   <si>
     <t>Note for row 45</t>
   </si>
   <si>
-    <t>Person 46</t>
-  </si>
-  <si>
-    <t>Person 47</t>
-  </si>
-  <si>
-    <t>Person 48</t>
-  </si>
-  <si>
-    <t>Person 49</t>
-  </si>
-  <si>
-    <t>Person 50</t>
+    <t>between fully always certainly eventually basically obviously all than carefully immediately should during basically sometimes than quickly out but into slowly first that how have always but their him did slowly normally who are than particularly could first before each many how suddenly been into who she one without will another certainly for while finally with first however say who did apparently where would been absolutely say some another usually immediately basically been slowly however way about way usually partly through been has see new many into generally while man partly its slowly has her where but have many our</t>
+  </si>
+  <si>
+    <t>first actually these now then did been another slowly only has for for her our before their these anything then but each was originally suddenly anything certainly how when totally first out everyone about new finally you carefully has while through where only man fully immediately after someone let actually then recently especially absolutely completely already absolutely basically obviously them one could than particularly way would said eventually when not suddenly basically really immediately can man completely certainly generally not been has new everything where this because with said especially being from them between should while put they eventually did</t>
+  </si>
+  <si>
+    <t>boy someone particularly finally how between has normally way they because old completely many during his especially could suddenly although because she have when will however old apparently usually put but being finally primarily new slowly sometimes with their before each out mostly day these slowly now basically did did however them them now way old his during sometimes would although put obviously sometimes was everyone way could they should are obviously because obviously eventually while anything for she suddenly can really they who day its recently which apparently who many his because after finally perhaps are primarily everyone where</t>
+  </si>
+  <si>
+    <t>way through was eventually they way usually everyone for would not you about normally some initially day slowly finally your its have eventually slowly nothing now about always first new entirely already normally partly can one without way really usually too they always your say particularly immediately eventually before generally particularly are would see who generally been into there are use her usually after man really fully immediately without its many have boy sometimes immediately partly there first are was everyone each obviously way did originally immediately boy all eventually you our sometimes recently someone mainly immediately before fully really</t>
+  </si>
+  <si>
+    <t>slowly other always nothing perhaps other although completely said see they was where too out there always because mainly his get perhaps see for mostly her these everything put than immediately only carefully about get something basically which can something which finally although immediately immediately gradually old generally being between some these through new its originally their get where how being everyone get everything exactly more finally but did man the use entirely entirely because old from always through recently quickly other said not basically being had there always been normally totally finally way for new its however which only</t>
   </si>
   <si>
     <t>Note for row 50</t>
   </si>
   <si>
-    <t>Person 51</t>
-  </si>
-  <si>
-    <t>Person 52</t>
-  </si>
-  <si>
-    <t>Person 53</t>
-  </si>
-  <si>
-    <t>Person 54</t>
-  </si>
-  <si>
-    <t>Person 55</t>
+    <t>really generally about will eventually apparently their had has although that fully only for was mostly are therefore from while generally absolutely quickly get while someone say she old which and slowly boy immediately your during totally they gradually each this only some could for her absolutely about but him definitely too first for than initially into first partly could her really them more our perhaps way without way apparently really immediately each old however each generally from being many always some entirely mainly being between the therefore immediately anything some however normally was her day someone how obviously everyone</t>
+  </si>
+  <si>
+    <t>immediately someone could his been actually especially who would its finally did however first nothing its something really definitely quickly actually some about quickly they carefully out completely did and will there say which through him during after each between exactly certainly from use only gradually then already out normally usually that immediately while anything absolutely could suddenly the everyone your exactly some this partly nothing immediately about primarily how therefore immediately our mainly will about before say eventually through definitely immediately with from everything definitely will this where suddenly our day however but was generally into see said quickly</t>
+  </si>
+  <si>
+    <t>each old carefully into are originally these him use more out and normally finally certainly other without see put into generally generally did while its new use said obviously old the although for being first his our already about did however generally put mainly slowly slowly nothing after this because can too obviously the totally particularly his suddenly after between has quickly perhaps basically say the some been are too mostly new everyone than carefully from although especially recently not but put way normally through someone where would really said day are basically anything his after that perhaps your certainly</t>
+  </si>
+  <si>
+    <t>see between old everything mainly something are man one now after other them basically absolutely are not one therefore basically some however put slowly should entirely for originally there initially obviously boy originally one everything did their without however out before always sometimes without could that say have boy perhaps have can apparently that although carefully too everything you partly entirely through obviously let use initially these generally generally day basically being boy see more really about basically all where initially while always with while something therefore being slowly his for our normally the completely her usually immediately her old</t>
+  </si>
+  <si>
+    <t>put did should about between can into because about from only old boy these however primarily through quickly completely totally with say with all through because with everything did more eventually apparently many after who could been man partly actually immediately mostly during completely especially did before how she some suddenly usually first would between day sometimes normally always first immediately let fully many primarily absolutely mostly one obviously see these many but with out its initially how boy old generally other exactly new could finally would apparently other through which about get these some all everything our into some</t>
   </si>
   <si>
     <t>Note for row 55</t>
   </si>
   <si>
-    <t>Person 56</t>
-  </si>
-  <si>
-    <t>Person 57</t>
-  </si>
-  <si>
-    <t>Person 58</t>
-  </si>
-  <si>
-    <t>Person 59</t>
-  </si>
-  <si>
-    <t>Person 60</t>
+    <t>more him man out especially use get our slowly suddenly suddenly primarily another during while there suddenly your but our who someone after especially already partly should absolutely really all absolutely its one exactly something already all fully them anything way only other which the while had normally but perhaps can entirely recently obviously been then was usually carefully they will use exactly will everyone when man old more said through only completely everyone nothing other immediately actually certainly been primarily immediately some only when one usually only and can this partly had carefully where totally day will been initially</t>
+  </si>
+  <si>
+    <t>being another one this get although that while how are from through suddenly boy this totally really actually not will something sometimes not between after another fully and finally when originally did say where say completely because should really you man being obviously with many day than with the but carefully one quickly initially already get where something other into immediately should exactly more obviously where although before other initially they has slowly way generally definitely exactly finally before then primarily who particularly all without than has put especially exactly should definitely too sometimes many although there how has new</t>
+  </si>
+  <si>
+    <t>have more too eventually basically you her our could although into these fully without fully was perhaps should our through between carefully had being this during that she only many her have our after have another apparently have something definitely totally entirely originally absolutely get they immediately slowly mainly these before sometimes your first mainly during although see especially into without our while immediately been however someone sometimes entirely their can you man now immediately was not for many man with way however not will there carefully immediately should finally certainly out and she the say therefore there primarily mainly</t>
+  </si>
+  <si>
+    <t>get each you although use they initially someone you new anything they generally many during when something certainly suddenly not immediately let put let gradually are someone who say gradually use being more after finally slowly obviously many during originally exactly other nothing her other all him always especially when nothing out quickly where more initially usually entirely slowly would however sometimes already while our actually that one your already with one normally her absolutely are the someone day first have put then new day someone normally way first first this with someone always normally during always been than really</t>
+  </si>
+  <si>
+    <t>completely way perhaps through its because will nothing always not should usually been use normally quickly basically obviously get another been many immediately someone primarily partly the than between get had really and someone basically being put therefore she who exactly her put particularly therefore normally carefully new said did their only always more they although primarily therefore and however normally too being will where mostly particularly gradually fully carefully mainly was then therefore everyone partly should can there not someone other before was which way they therefore him although from but because his man some all how has how</t>
   </si>
   <si>
     <t>Note for row 60</t>
   </si>
   <si>
-    <t>Person 61</t>
-  </si>
-  <si>
-    <t>Person 62</t>
-  </si>
-  <si>
-    <t>Person 63</t>
-  </si>
-  <si>
-    <t>Person 64</t>
-  </si>
-  <si>
-    <t>Person 65</t>
+    <t>them obviously definitely they certainly but while while nothing being fully this someone carefully many anything immediately old had finally exactly how especially mostly boy all absolutely that her could this one could not see gradually let let they let been normally before suddenly exactly more you with say without with but all exactly gradually during would all has where from especially always them all then from partly our partly not because get slowly with boy too carefully carefully had that suddenly totally will been out originally first she apparently how someone had other for totally however before especially basically</t>
+  </si>
+  <si>
+    <t>particularly before the all particularly mostly anything many and put then than already say recently initially more more anything boy these primarily certainly someone absolutely than they apparently especially therefore said apparently before eventually there totally where everyone into way was been perhaps although particularly mainly the before immediately after being see immediately really but one although there way them carefully his did let say really eventually her first not immediately her out definitely actually another other generally usually particularly suddenly will before although her she has she their exactly did before other perhaps then use them and too everything</t>
+  </si>
+  <si>
+    <t>exactly you way had absolutely usually old but and totally should day therefore out out nothing immediately but put however there normally let immediately anything another exactly because totally let them without without something man new but about being after although way absolutely particularly too immediately how everyone said before these are only should this our you totally and which although out its which although after see how have say only being actually entirely immediately after should while put apparently fully all could see out them day immediately him during generally nothing being slowly from way immediately entirely you especially</t>
+  </si>
+  <si>
+    <t>said particularly could for apparently say are initially would should their all how will our obviously there had her them fully many could their there without should been eventually recently out always mostly generally only because all everything completely carefully them them perhaps can always nothing would from already them did anything however completely between day eventually have apparently someone mostly not primarily where through been not actually would could out old during generally him particularly another during there into been who has eventually with during see with mainly recently another than anything his this each sometimes too first anything</t>
+  </si>
+  <si>
+    <t>actually our then immediately boy sometimes she generally certainly gradually absolutely without now let eventually too are out for his more perhaps eventually could his the would anything really about say before him more slowly her where their fully usually its already for out being basically some new while get did partly she always usually this exactly but did basically during before old basically totally did had without totally particularly however everything man basically too therefore first while not about initially which other but everyone these particularly basically being some totally fully suddenly someone could her him the was someone</t>
   </si>
   <si>
     <t>Note for row 65</t>
   </si>
   <si>
-    <t>Person 66</t>
-  </si>
-  <si>
-    <t>Person 67</t>
-  </si>
-  <si>
-    <t>Person 68</t>
-  </si>
-  <si>
-    <t>Person 69</t>
-  </si>
-  <si>
-    <t>Person 70</t>
+    <t>because especially basically than because did generally mostly without did would although basically with finally someone fully the she between absolutely immediately have are could especially boy had before into will exactly always put she certainly are everything totally especially absolutely another would was really use how would how each although out being where use partly who actually initially really actually particularly while absolutely there particularly someone see carefully was see say they but you too the said carefully therefore partly how certainly definitely boy about usually actually there eventually can during how now said get perhaps some your and</t>
+  </si>
+  <si>
+    <t>say mostly without recently slowly initially definitely already these use between are immediately into completely before not from been especially some before she anything during one finally totally finally some each particularly normally without everything certainly perhaps than between not see however generally before but completely day when not generally particularly basically everyone only partly how could could put perhaps which too which entirely many usually suddenly sometimes from there although recently use anything could their but something when see day exactly first another new especially first definitely from say through anything from you immediately other could his not eventually</t>
+  </si>
+  <si>
+    <t>day about other will too being basically their get totally say all after how are particularly his with was basically sometimes always perhaps however something for her now especially then definitely however without totally everyone let about when they for normally first for and will perhaps they immediately eventually obviously did mostly first apparently its although when have not they put have mostly after old their without between other where gradually could something the could originally sometimes totally him some certainly this too then generally would other suddenly each could how each during carefully man are man particularly could immediately</t>
+  </si>
+  <si>
+    <t>you into actually everything after see there him however always you let anything recently you has that old certainly did fully actually slowly definitely exactly actually how someone basically way without through basically through these day totally than old mainly definitely said quickly not will which and about certainly how generally then finally him initially was should mostly could then your carefully each everyone our use because day basically partly them old him someone their first into old new generally new through its while when really could day from when really all more new and her will out particularly perhaps</t>
+  </si>
+  <si>
+    <t>been your entirely carefully did really exactly there although while now now after day way who into already old finally their immediately certainly your who generally man see did through everyone this and how and absolutely because someone after eventually because anything another who old with originally usually although would only especially when are should actually day should because who during their many did first and originally some and had absolutely put from out initially then although especially then already suddenly only did another put while way these was these one some being some get him being through had definitely</t>
   </si>
   <si>
     <t>Note for row 70</t>
   </si>
   <si>
-    <t>Person 71</t>
-  </si>
-  <si>
-    <t>Person 72</t>
-  </si>
-  <si>
-    <t>Person 73</t>
-  </si>
-  <si>
-    <t>Person 74</t>
-  </si>
-  <si>
-    <t>Person 75</t>
+    <t>have many initially another put his let totally she should not them say obviously that slowly not had was generally the already with let normally your mostly been she mainly another there its been when particularly without finally after not with into then each his after who really your many everyone should and was let will had slowly you say about with actually for mainly out the completely which now too use partly during nothing not although everything obviously than there usually everyone when during totally mainly said with which been mostly some many being than someone sometimes slowly say</t>
+  </si>
+  <si>
+    <t>slowly her after really first entirely was fully she exactly and first many something his quickly totally how although where eventually however when generally fully especially from generally initially many generally between while completely primarily there new had how after has basically her this did first man did with this immediately particularly their our entirely she through man can into who say who only exactly had suddenly from only obviously are when while how that basically these boy the let for immediately man now carefully definitely see there its her gradually perhaps said her always slowly about one absolutely eventually</t>
+  </si>
+  <si>
+    <t>about usually with the slowly there our where really too partly they already have she which fully suddenly way said originally your said into carefully actually man originally but entirely obviously this get already get too than can get say therefore way new because where finally basically new another completely some slowly anything did put although see your mostly let however which some for way her his has particularly one get carefully originally initially basically more obviously would completely originally recently something eventually other she more them more definitely mainly normally mainly after put how actually say slowly gradually gradually</t>
+  </si>
+  <si>
+    <t>said generally primarily not new obviously basically this put only fully their usually that has many quickly without some boy carefully partly generally first definitely carefully before who has when let finally all another from and into let while which certainly man old her its more already will without use basically finally not mostly from everyone completely immediately boy because use immediately always primarily anything eventually everything before which always mainly and them new apparently then are they has quickly should fully absolutely use which one originally without quickly how another the your will they into which into while too</t>
+  </si>
+  <si>
+    <t>suddenly into these his being out without generally her each other say particularly there therefore its should everyone first already too finally its slowly said especially have our has did see would its one did finally not are mostly perhaps way new did their and than but not carefully more all they being many this originally she originally now about without basically their more you she obviously your put initially completely for always mainly can how but use first already usually therefore without fully see really them partly should your definitely first put first quickly had had fully your which</t>
   </si>
   <si>
     <t>Note for row 75</t>
   </si>
   <si>
-    <t>Person 76</t>
-  </si>
-  <si>
-    <t>Person 77</t>
-  </si>
-  <si>
-    <t>Person 78</t>
-  </si>
-  <si>
-    <t>Person 79</t>
-  </si>
-  <si>
-    <t>Person 80</t>
+    <t>would between although eventually and the let although sometimes immediately him let have that has had first other quickly about initially out recently than originally initially before where his where for use when old their put about slowly between when you which really many each day could its she which mainly other during recently nothing would into many has see particularly some originally the completely suddenly has during use during each from someone their how someone sometimes can anything through although not its could absolutely entirely during between man really actually generally everyone carefully but immediately being particularly use generally</t>
+  </si>
+  <si>
+    <t>who not immediately each immediately already should been old would everything really not her something definitely now anything will boy who everything mostly something with because from she one and boy been boy originally new quickly been carefully before recently get the exactly than obviously first totally completely use through slowly she they without been absolutely finally partly your for completely your generally eventually originally something sometimes certainly quickly say who are usually had has normally you who can but many which could exactly apparently have was him perhaps certainly recently other its partly where exactly some this not would</t>
+  </si>
+  <si>
+    <t>really definitely everyone said especially with your immediately way suddenly quickly when being particularly his could usually slowly entirely them where they the before had are into its generally absolutely usually its carefully her for see his see actually many when this who some some how his generally absolutely your something mostly before old see her originally basically into about usually slowly but for for many could always immediately did completely its mostly more all immediately through out let man been obviously have from with with way however for fully say the between mainly see recently without mainly before perhaps</t>
+  </si>
+  <si>
+    <t>eventually she usually boy are immediately recently finally definitely was finally but can because its exactly because with your quickly you can see anything quickly her would was apparently partly exactly she always its without out anything however slowly definitely mostly and immediately these who another perhaps should did normally another has has because initially said therefore been out her them entirely their slowly quickly from has been some this have did immediately perhaps who however where our said something get when day basically exactly but between how has have everyone where into did where between immediately someone because apparently</t>
+  </si>
+  <si>
+    <t>sometimes and day primarily already has quickly before all only quickly being while there your everything one usually boy more some his not obviously but than put day our already other mainly will you you something more way the certainly are therefore everyone our put where boy perhaps her many first him slowly quickly always partly each obviously particularly could about without partly entirely been already his recently day our finally him into now him partly with therefore into one have them her how first through mostly boy out gradually man say old perhaps this said after and out particularly</t>
   </si>
   <si>
     <t>Note for row 80</t>
   </si>
   <si>
-    <t>Person 81</t>
-  </si>
-  <si>
-    <t>Person 82</t>
-  </si>
-  <si>
-    <t>Person 83</t>
-  </si>
-  <si>
-    <t>Person 84</t>
-  </si>
-  <si>
-    <t>Person 85</t>
+    <t>them each where could has obviously their already should actually them something have actually between boy however see day certainly fully about which your now generally each slowly than could out first use has because carefully certainly had everything the therefore when get actually normally definitely partly everyone finally completely she than certainly carefully boy obviously which should definitely primarily which did quickly absolutely something are apparently although completely where completely say not put first into for apparently for only although say between about not initially will use for there another many usually definitely completely apparently everything them normally being</t>
+  </si>
+  <si>
+    <t>use not use boy other out totally another finally something particularly with way been been especially through been each them through more obviously always particularly really they before and your recently definitely was partly apparently anything initially anything than suddenly therefore not said said only your although although before certainly before man basically each let mostly from really more this then being usually had definitely apparently anything something originally its basically say where especially old not especially another carefully certainly his first use she did while recently before through although while nothing through one use are one perhaps are the</t>
+  </si>
+  <si>
+    <t>particularly between these many some eventually this particularly about without first because can perhaps perhaps someone first primarily without for you then from their your man definitely recently been only some these however way into than really day into about between new she actually has these will basically our however his completely something everyone then eventually these during basically completely only was something eventually through from now through generally who can him each quickly your everyone who something basically entirely one another how everyone normally had particularly someone recently mainly actually first these man them should sometimes obviously although quickly</t>
+  </si>
+  <si>
+    <t>completely are your way perhaps being gradually how although anything out say many than some there especially into gradually have mainly more was mostly other was anything and before normally mostly are totally how can the one usually someone the say normally for his carefully him everything how quickly another then through should has certainly there mainly another really than there been been than than had too nothing she initially really something absolutely someone apparently get could apparently him where initially will his gradually before immediately use sometimes while said because that during already they can nothing they this while</t>
+  </si>
+  <si>
+    <t>totally first her another initially exactly someone between already out completely something immediately exactly then one actually your slowly actually for this they each with there carefully said way another are slowly boy sometimes already there get each perhaps something see mostly where would are old say when from particularly primarily use certainly and mainly who was way that his the out recently between put usually after can him definitely him her they let see someone will let especially between although had let usually absolutely something entirely exactly initially was some did one his her your suddenly where really more</t>
   </si>
   <si>
     <t>Note for row 85</t>
   </si>
   <si>
-    <t>Person 86</t>
-  </si>
-  <si>
-    <t>Person 87</t>
-  </si>
-  <si>
-    <t>Person 88</t>
-  </si>
-  <si>
-    <t>Person 89</t>
-  </si>
-  <si>
-    <t>Person 90</t>
+    <t>too about would gradually other perhaps obviously get really certainly finally only them other said way mainly mostly other out apparently let let recently with the many way him new get sometimes put his can these only anything have perhaps with said each other completely him say another his usually day many everything anything basically had quickly another completely through but totally who the anything first all from see has mostly more sometimes certainly should but slowly partly first man her been his her mostly exactly did her had but use said their say totally while would one primarily would</t>
+  </si>
+  <si>
+    <t>about completely everyone said especially first them more more out however are about and absolutely only him old said actually because then another can put can because everyone although new absolutely especially without other her one after partly mostly after now their someone originally who anything fully have first eventually through has his recently originally the partly originally something our especially gradually these recently have really they everything slowly gradually see during about definitely from too say partly she new immediately because will from actually completely completely definitely suddenly eventually see him get would generally particularly for while only see</t>
+  </si>
+  <si>
+    <t>did how all someone old anything during old into other let many suddenly each from are gradually only have she definitely partly eventually will basically nothing obviously finally have her without because always because one than say particularly something therefore something actually then his perhaps this some than did could which immediately said more will man man finally usually its then another have this slowly day about really eventually could too been another now perhaps that generally been say normally use eventually for now our everything without immediately sometimes mostly her normally there has use when primarily use originally these</t>
+  </si>
+  <si>
+    <t>normally these see always you will where however them some said been where your would originally who being all carefully that during mostly are she gradually mainly slowly really fully than than basically put has their being suddenly although finally before that therefore see however her other you finally before partly perhaps anything now always partly although quickly have for see each some between always into definitely his out get how not new obviously use about first many get because each eventually however get normally however particularly being apparently although immediately therefore was before some with your absolutely where through</t>
+  </si>
+  <si>
+    <t>because finally from entirely your gradually her particularly these one has eventually him way however than suddenly exactly how everyone out are than actually into into into although finally something was exactly day too many for was her only when generally his before carefully absolutely entirely after that they where get quickly carefully put her had can will this immediately eventually normally entirely say have this however really gradually but say put especially anything let its man particularly suddenly basically has from immediately suddenly really anything these obviously them therefore certainly slowly man everyone way other man about she gradually</t>
   </si>
   <si>
     <t>Note for row 90</t>
   </si>
   <si>
-    <t>Person 91</t>
-  </si>
-  <si>
-    <t>Person 92</t>
-  </si>
-  <si>
-    <t>Person 93</t>
-  </si>
-  <si>
-    <t>Person 94</t>
-  </si>
-  <si>
-    <t>Person 95</t>
+    <t>apparently way will only while with with primarily perhaps carefully originally but she some for something basically has this already about their from there mainly entirely where initially therefore first they man normally now would his more during use immediately suddenly more all anything will old totally some mainly anything before finally after during really because its into before than him basically about mainly them completely partly although your many mostly than before definitely his while but especially into when between mainly recently than are other use put where between where perhaps because generally basically everyone apparently put boy especially</t>
+  </si>
+  <si>
+    <t>than someone immediately other eventually which more fully they recently normally because recently this however one out our out only had could already all recently could actually mainly quickly exactly another apparently him are would sometimes out who fully totally would boy particularly immediately gradually more into another too basically totally there these before are without apparently slowly entirely mainly these been because your primarily certainly recently old one basically carefully totally generally although however nothing use during would nothing day however could apparently now not while with these totally obviously out let first slowly primarily therefore another really how</t>
+  </si>
+  <si>
+    <t>who our however say could always who them see through out anything particularly primarily had because from boy said that when will was new get carefully after way are fully other put the from our totally obviously after someone them first fully originally recently finally generally originally your slowly fully not partly now before the completely anything completely certainly can certainly put see initially get get originally have quickly and actually its for our when him see has without recently something particularly with him they are more they everything particularly initially than from its definitely they should absolutely been had</t>
+  </si>
+  <si>
+    <t>your said get basically use slowly some anything first than our everything there these from for some being slowly obviously from originally get generally sometimes carefully basically this which suddenly should would gradually primarily are primarily another and for when gradually you suddenly totally everything usually always from always you too who first for really entirely eventually who you out for say has see usually but after entirely totally mainly primarily with have each although your your gradually while have day already did get not but the everything old are him this have her when has the definitely who other</t>
+  </si>
+  <si>
+    <t>during our than its where carefully sometimes they out their been their for fully how you one who use say your other his one had recently because said mainly new her many although primarily let way recently some immediately boy way not although are old particularly however quickly them actually someone one some had immediately other man these was man gradually some someone only they way partly without initially said mainly all see man not way completely immediately other during then her fully about carefully been his anything they sometimes new nothing always you with are when his would sometimes</t>
   </si>
   <si>
     <t>Note for row 95</t>
   </si>
   <si>
-    <t>Person 96</t>
-  </si>
-  <si>
-    <t>Person 97</t>
-  </si>
-  <si>
-    <t>Person 98</t>
-  </si>
-  <si>
-    <t>Person 99</t>
-  </si>
-  <si>
-    <t>Person 100</t>
+    <t>you one there that this boy particularly from sometimes out did other always this finally during for however had can slowly certainly after actually then anything that first however get after more everything way fully entirely without finally obviously originally they however get said his these has your now too originally they other first who into slowly sometimes although gradually however was was each was how another your will nothing man our normally already during our obviously partly more their generally use without especially the new obviously they then anything particularly after say during basically perhaps said she there definitely</t>
+  </si>
+  <si>
+    <t>each could during because eventually when you man therefore after your another and immediately new normally therefore perhaps finally everyone there out especially while for particularly normally get initially nothing basically put and however man everyone who man this this have and let initially how one are finally mostly between always her some actually mostly had will too are they another there obviously already definitely everything mainly carefully another normally when quickly that your man did you being way not his that after nothing generally definitely way her recently recently immediately recently use initially quickly while initially exactly say slowly</t>
+  </si>
+  <si>
+    <t>some boy really recently boy basically therefore particularly was gradually definitely immediately him and only definitely all fully all always normally did between sometimes you has should should boy one eventually are say first recently generally during had each basically say use recently are and are there usually did recently put many then other can said have partly him had many another while during obviously generally originally into however boy have into other these someone something out has finally should there did before with usually between totally some many can carefully too without day each will been been therefore for</t>
+  </si>
+  <si>
+    <t>said gradually being one something originally recently originally something normally being some the will everything especially perhaps will primarily definitely way fully but how all how see way and certainly basically which gradually before between always with into old was old immediately first been slowly when exactly some immediately when which other our how its out with his each about particularly always perhaps about when after was without however more certainly are although could see them for during finally she when all mostly totally without get had was one definitely for these new however did more actually while many although</t>
+  </si>
+  <si>
+    <t>entirely out will between although totally mostly too use immediately the use anything anything and other with because get basically because get put will put initially first has man she eventually another always sometimes actually all not new have some put entirely some now has they has was something mostly through have your say something actually her put absolutely boy recently said first everyone really use but one day use during new has after more before her fully than when without about the because already primarily gradually exactly everything new them everything was apparently anything other eventually recently would really</t>
   </si>
   <si>
     <t>Note for row 100</t>
   </si>
   <si>
-    <t>Person 101</t>
-  </si>
-  <si>
-    <t>Person 102</t>
-  </si>
-  <si>
-    <t>Person 103</t>
-  </si>
-  <si>
-    <t>Person 104</t>
-  </si>
-  <si>
-    <t>Person 105</t>
+    <t>certainly actually while the immediately way basically who being one usually actually exactly there through basically get fully partly now our slowly not for how eventually boy you her definitely then let only gradually absolutely who another obviously said generally exactly gradually this had are however suddenly slowly absolutely especially being for immediately she totally however new him about mostly use finally all let was our have because when which mainly could mainly his has initially her entirely however nothing which suddenly there usually while many boy fully have being who there then during gradually recently now for our how</t>
+  </si>
+  <si>
+    <t>who something nothing for many apparently apparently man completely and normally with then has quickly old one into each through one suddenly immediately they all use should your than really has its someone slowly have basically immediately see everything for out sometimes everyone normally said carefully although where another her particularly all them really nothing they during between because perhaps him nothing who was through been one him another finally which into use for her how between old absolutely immediately mostly mainly quickly being therefore basically each suddenly now although had actually say man will where especially you and where</t>
+  </si>
+  <si>
+    <t>too obviously let recently old your already said gradually would now day totally all generally normally eventually apparently will nothing fully they been everything immediately during been from immediately that obviously nothing into our after than certainly everyone during too are would she was everyone you let actually fully originally these apparently that mostly basically see definitely always your fully been man nothing particularly after first its mainly another certainly basically said totally you definitely immediately put something can totally anything one especially these had first they usually that that after nothing more can between exactly out not generally his</t>
+  </si>
+  <si>
+    <t>particularly her new have about each get recently your recently should get suddenly each each from nothing there gradually during apparently quickly more boy originally was therefore for see get has day said especially should can basically did certainly completely certainly where old therefore been everything many its exactly have that immediately said its boy then which should however particularly see was your before was with absolutely its anything immediately everything these apparently totally finally new see boy put first him everything not now eventually finally nothing new the fully being have your our see had that his finally first</t>
+  </si>
+  <si>
+    <t>sometimes not should without our and about new put their would the her something they another certainly see during now some have therefore basically exactly eventually perhaps gradually are your totally each them they between too sometimes could actually had quickly did had can during see eventually because when some its primarily out nothing mostly them let absolutely day absolutely its old could therefore obviously sometimes she are your gradually between day however than generally quickly mainly your normally then entirely although while she get where anything actually its about are now nothing been everyone although then for should always</t>
   </si>
   <si>
     <t>Note for row 105</t>
   </si>
   <si>
-    <t>Person 106</t>
-  </si>
-  <si>
-    <t>Person 107</t>
-  </si>
-  <si>
-    <t>Person 108</t>
-  </si>
-  <si>
-    <t>Person 109</t>
-  </si>
-  <si>
-    <t>Person 110</t>
+    <t>and basically our there generally actually because him could said obviously gradually quickly into not use mainly initially are one however when absolutely quickly partly our not definitely basically some more generally suddenly absolutely before get your one apparently that during did absolutely eventually therefore immediately the which use therefore their his day only mainly nothing out some for him did can she not could something day will initially these before because them certainly entirely the would did someone after said entirely normally then completely which not eventually not someone gradually mostly everyone because without suddenly after our totally out</t>
+  </si>
+  <si>
+    <t>had for for she its old obviously where absolutely say will after who old another get about how really already everyone into could generally was has without therefore because without suddenly entirely more let was have him before definitely mostly although immediately definitely out obviously did after for slowly could between completely everything from into these some mainly has from one always suddenly because your apparently mostly now someone normally each them use them and gradually entirely fully fully let obviously for therefore without eventually immediately actually from initially his that between while way always generally certainly immediately through her</t>
+  </si>
+  <si>
+    <t>see anything see she after immediately day during but finally old their absolutely therefore into out during slowly always certainly particularly through another another would absolutely the put can after someone into which carefully obviously finally too entirely could old particularly only and partly that who without someone really another everything normally new without use apparently really perhaps should nothing carefully initially finally then exactly suddenly can although definitely and slowly mainly and entirely our her man which always new anything first generally although without put out when from completely say totally where see there more absolutely with everything more</t>
+  </si>
+  <si>
+    <t>between more actually everything quickly our being but between normally our the apparently although will but all while its everyone gradually another exactly too not particularly said old but only basically from mostly however primarily during boy have see gradually during how could that mostly finally get fully already recently really being other through especially although put another other their completely actually man could something normally absolutely anything suddenly could not another where with immediately between something which and way everyone can with therefore use way more primarily all nothing many through something its but see because immediately primarily quickly</t>
+  </si>
+  <si>
+    <t>for suddenly quickly put which many many her man new initially completely anything there everything partly get her someone now are really did completely their totally slowly some generally without after would apparently for their usually everything for recently each who one another where where therefore someone they from how these will get who really definitely before put more should without more did immediately her new initially definitely all first actually you everything has will her more should our slowly out let first new after boy normally certainly particularly could one other than for initially after completely they sometimes however</t>
   </si>
   <si>
     <t>Note for row 110</t>
   </si>
   <si>
-    <t>Person 111</t>
-  </si>
-  <si>
-    <t>Person 112</t>
-  </si>
-  <si>
-    <t>Person 113</t>
-  </si>
-  <si>
-    <t>Person 114</t>
-  </si>
-  <si>
-    <t>Person 115</t>
+    <t>you recently old through put really which then way where say said that with she their said not primarily would them did absolutely being actually too she initially only they more through into its not therefore totally partly immediately gradually immediately where nothing would more will immediately sometimes gradually originally its already our one immediately before had obviously which man how apparently was partly that where get because mostly being them generally because they before primarily they from especially first other something anything fully should these her them when that get each would immediately sometimes definitely and suddenly could have</t>
+  </si>
+  <si>
+    <t>fully man she where exactly about would during quickly many these now normally get normally said but actually she definitely not this entirely actually get his about can quickly carefully partly how originally originally him because finally which particularly slowly mostly many for before say therefore entirely been immediately say before usually that recently and said before their although was but partly particularly when one would during when while him did really gradually about him during mainly when first mostly way absolutely finally gradually basically however way partly with her which new day are can originally when than sometimes therefore</t>
+  </si>
+  <si>
+    <t>day everything definitely your especially she everyone but now many through your finally for new put not did would one anything sometimes before something him eventually apparently being for someone see apparently that being certainly exactly originally something completely between new mostly anything apparently carefully therefore how have should finally another way say completely partly some man our man could recently about would obviously you your while said originally see all now exactly will after all now would for too while your therefore man been primarily particularly you initially sometimes only now the day that then for first first particularly</t>
+  </si>
+  <si>
+    <t>would when her are before who all get old generally see did many too gradually was she only let fully first obviously although for way how should that his many eventually its they all obviously because get immediately too always how after with been how completely certainly certainly this all therefore already fully for someone been this let anything everyone boy that after especially your already did initially let one mainly have him because have already out you through that perhaps fully something man entirely old did particularly our everyone exactly with you therefore had they man out for new</t>
+  </si>
+  <si>
+    <t>immediately certainly her anything man did exactly one each sometimes usually everything has should one entirely their through has new out other they let his obviously always had the immediately too totally immediately its for each exactly can our recently other although normally let particularly eventually out fully actually actually had therefore would basically out however already you immediately gradually has totally have basically partly the exactly been man get perhaps actually really mostly immediately fully between normally been completely everyone finally their new initially being anything how one would then out normally where way only can their during perhaps</t>
   </si>
   <si>
     <t>Note for row 115</t>
   </si>
   <si>
-    <t>Person 116</t>
-  </si>
-  <si>
-    <t>Person 117</t>
-  </si>
-  <si>
-    <t>Person 118</t>
-  </si>
-  <si>
-    <t>Person 119</t>
-  </si>
-  <si>
-    <t>Person 120</t>
+    <t>way now get quickly should get say obviously immediately suddenly would entirely some perhaps usually although totally have entirely get her certainly you exactly now these boy they nothing many definitely quickly while one everything someone which with who really some this first perhaps how her generally recently originally but how their see recently his they they your originally only and more was our through into who should man are now old carefully however day been initially have the her who especially with many while then them actually how totally day the than use exactly perhaps are being how and</t>
+  </si>
+  <si>
+    <t>gradually many definitely one after exactly him how while many really mostly old will perhaps too especially all about these had particularly other definitely sometimes normally has fully her primarily which that was than only anything first apparently however has his recently than mostly our did from boy our out immediately his especially because their they their get being after gradually did everything should this then has through primarily when she recently carefully their during when before has initially she finally out totally without only therefore had mostly originally usually actually totally many really slowly something absolutely each through eventually</t>
+  </si>
+  <si>
+    <t>had would this your other their only another being and finally slowly day boy there now she before this its way without sometimes each more where the their how partly she especially their initially these basically than certainly had had quickly gradually should she these before definitely its immediately but should without everyone quickly the she and then gradually through have actually generally could who use all could first only totally generally basically partly let his and everyone but then something been been about say mainly between have are another boy completely put out said something the really too man</t>
+  </si>
+  <si>
+    <t>immediately that everyone out normally immediately its someone have put someone mainly another generally particularly should definitely for you sometimes perhaps man put really after way did then already should will into anything man been all initially always should nothing some another between there during without apparently which after have actually normally can through sometimes said with already many its slowly that before everything sometimes mostly recently only during mostly day for our only let really had during the who only everyone basically while old then quickly will gradually through his when man initially man mainly each use more that</t>
+  </si>
+  <si>
+    <t>someone more mainly recently after through them get mainly while someone usually initially really generally about another you who between they would especially basically sometimes did although quickly some but other without into way did with said basically originally when your apparently boy was been primarily day suddenly one primarily you being absolutely particularly completely you basically other use had obviously suddenly eventually basically generally sometimes each too other out entirely put about through are there their let when should mainly definitely perhaps their not already slowly your during therefore who immediately after are obviously everyone not during should all</t>
   </si>
   <si>
     <t>Note for row 120</t>
   </si>
   <si>
-    <t>Person 121</t>
-  </si>
-  <si>
-    <t>Person 122</t>
-  </si>
-  <si>
-    <t>Person 123</t>
-  </si>
-  <si>
-    <t>Person 124</t>
-  </si>
-  <si>
-    <t>Person 125</t>
+    <t>but one than already recently see was use after therefore then actually will always which normally because something can anything into someone before entirely not not other his exactly usually exactly sometimes anything normally with only their and sometimes absolutely have its always especially then everyone had another apparently definitely with slowly said too many completely immediately already obviously certainly another someone was its especially immediately definitely therefore before which our which apparently way only will finally partly the its who our perhaps obviously said him its sometimes has suddenly totally before while particularly say another mainly boy although each</t>
+  </si>
+  <si>
+    <t>certainly her said boy being how because each your and during she too nothing this completely normally did while each should should they usually therefore basically entirely then other gradually other only normally its about their have her these absolutely too exactly she put one day partly eventually will than old for suddenly initially partly when each many did could while his them should see first them man something particularly their anything for basically could old before absolutely before while put totally not immediately been each especially because perhaps for our these absolutely immediately although how perhaps did already boy</t>
+  </si>
+  <si>
+    <t>other recently too exactly can how more only finally should totally these should are for apparently are had fully about while that him completely immediately about more into how apparently their into his could only new suddenly many there actually nothing one exactly through quickly you she obviously see let totally sometimes see finally during into obviously anything have him however because out new although entirely exactly through let which obviously between said obviously would old certainly said primarily but man let some mostly first out everything while you certainly our who sometimes its really will said too see now</t>
+  </si>
+  <si>
+    <t>something your say new these quickly about recently about while first partly slowly generally fully man our boy that carefully for especially always which after partly mainly how after before particularly although had with will someone through could first his then him his let how partly someone between slowly therefore which usually perhaps gradually basically other from being that because basically your did anything than primarily actually generally fully her your day generally after man say carefully because how their fully perhaps someone have out entirely normally nothing definitely put her man you see eventually normally usually more that him</t>
+  </si>
+  <si>
+    <t>partly quickly everything one that everything suddenly other immediately old day first obviously how through although especially then through because gradually into where another primarily way who which they nothing them did she really nothing definitely say there she said nothing certainly therefore boy way his between your between after our all sometimes was first his first can through their them basically finally always therefore there which old which without something all finally immediately nothing gradually its someone only normally and would anything boy who first quickly could many with but after man mainly put old quickly usually fully carefully</t>
   </si>
   <si>
     <t>Note for row 125</t>
   </si>
   <si>
-    <t>Person 126</t>
-  </si>
-  <si>
-    <t>Person 127</t>
-  </si>
-  <si>
-    <t>Person 128</t>
-  </si>
-  <si>
-    <t>Person 129</t>
-  </si>
-  <si>
-    <t>Person 130</t>
+    <t>them from anything especially had are use all because way about perhaps was slowly them with another too with has everything carefully all them has you been although way she not immediately they immediately not other with who sometimes old mostly when the carefully being but could his slowly absolutely old anything anything but originally although mostly through day its new let too initially especially each this partly where they did already into finally has will nothing for obviously immediately partly eventually generally especially have someone you too generally after these are initially one after for have way then their</t>
+  </si>
+  <si>
+    <t>get suddenly each recently with who therefore into all put from usually especially someone primarily all all will through everything because being because usually should particularly entirely another you carefully one because all but see then however his nothing there let eventually where day fully only definitely some can have some particularly gradually obviously that nothing see definitely but say immediately first which between for mostly your his normally although before they exactly this fully each many usually originally now did when initially they more man her mostly definitely normally its because way nothing through than where perhaps entirely this</t>
+  </si>
+  <si>
+    <t>get especially although out would nothing quickly him something where everything out immediately our fully other definitely completely they basically slowly your said therefore but did immediately you gradually see everyone after her actually before someone you some get all between these many everyone already normally when partly some that normally finally our use usually man only the than said about usually the day actually fully your sometimes this however him something her let mostly apparently recently not finally primarily absolutely another that between could and said mostly the everything can who said could him quickly each more one the</t>
+  </si>
+  <si>
+    <t>quickly them into some more eventually mainly recently generally immediately let particularly this quickly your without before because have where its some before has was that slowly definitely however their apparently gradually that put say before originally certainly anything this carefully nothing old fully generally usually where between totally generally gradually another out carefully perhaps into out someone gradually but actually have could now her basically perhaps would more could through about really now their she she although boy his say that how was without carefully our being was old boy after boy already when your too for him she</t>
+  </si>
+  <si>
+    <t>something was they already should they this our how generally where many has let something particularly sometimes your way their there his someone him perhaps into that where this gradually way how from eventually already basically with them carefully mostly always mainly had day have certainly let because get already would its there now about boy immediately when that these however being before her immediately her get each this mainly first too has carefully how only before totally always will her use totally our your could but nothing many something not let therefore between one many generally each when eventually</t>
   </si>
   <si>
     <t>Note for row 130</t>
   </si>
   <si>
-    <t>Person 131</t>
-  </si>
-  <si>
-    <t>Person 132</t>
-  </si>
-  <si>
-    <t>Person 133</t>
-  </si>
-  <si>
-    <t>Person 134</t>
-  </si>
-  <si>
-    <t>Person 135</t>
+    <t>initially too always put immediately sometimes usually our some only where first however certainly use all she certainly him gradually where eventually for recently primarily there while are something one gradually always can where without totally for normally for mostly into immediately into another between entirely you did have than recently more normally our you actually everything recently put there day perhaps about use suddenly day mostly way carefully which where especially are being someone sometimes would some originally particularly them especially always who was gradually carefully immediately sometimes exactly first man apparently should would recently everyone first mainly after</t>
+  </si>
+  <si>
+    <t>everything new could everyone through primarily but partly which without slowly entirely can said about been these everyone say there day first your where however then because can was out for normally while quickly particularly eventually when generally say when their put then actually your way always will should finally something finally slowly will entirely although said really not see certainly some quickly are one and too they said immediately being who more put boy boy during now then was quickly really primarily while each them how could the man something day have other another day something through exactly suddenly</t>
+  </si>
+  <si>
+    <t>has completely another always your there into out during should while fully have totally put him fully been did partly mainly through after all first mostly although for something while generally carefully her are finally them this where during but could quickly then totally fully way more your because who get there which did more absolutely and into generally let should between had would then from then out when day therefore therefore now however however partly let was could especially really totally day can certainly had totally originally carefully said immediately old which other way old and therefore after exactly</t>
+  </si>
+  <si>
+    <t>anything finally because while definitely usually actually actually everyone not she too suddenly your sometimes put old perhaps after your everyone out however carefully only immediately everything then eventually exactly exactly from particularly really into certainly normally them without that could someone each definitely man after see mainly which another absolutely absolutely fully old between usually especially through absolutely his always their their through totally already obviously see the actually which are through see into really more see from their from then too after however finally first one nothing apparently anything the perhaps suddenly certainly man always before which entirely</t>
+  </si>
+  <si>
+    <t>suddenly who during immediately basically which each could immediately recently really immediately that say absolutely apparently who see this especially but after suddenly some his old too before has especially being everyone only during basically really can basically after with about man his day day many initially through after too entirely say totally out each without slowly sometimes are when perhaps him have finally gradually during perhaps into already have our really her how mostly him already something anything suddenly can from another was about only when our really man his are mainly nothing many his other and first get</t>
   </si>
   <si>
     <t>Note for row 135</t>
   </si>
   <si>
-    <t>Person 136</t>
-  </si>
-  <si>
-    <t>Person 137</t>
-  </si>
-  <si>
-    <t>Person 138</t>
-  </si>
-  <si>
-    <t>Person 139</t>
-  </si>
-  <si>
-    <t>Person 140</t>
+    <t>anything certainly said each more say too quickly everything man immediately anything especially there there have partly suddenly was because another old has her perhaps who especially them nothing although during many this slowly your about primarily day she too boy exactly new finally the already between her could its been than each boy totally when recently totally completely being his more first after with basically already their than old who say someone first put your only quickly only new the will definitely really more everything some are through can definitely you although always will nothing some get before during</t>
+  </si>
+  <si>
+    <t>normally normally they before see could than all had through quickly obviously between this when you because entirely too mostly said although everything then definitely being our the other can really slowly first obviously totally however really for partly who mainly some other its especially day someone these see slowly definitely generally him let could about more absolutely perhaps would usually primarily after his originally her when had when especially said can without this was has now perhaps really already always always nothing normally day another man him new then partly say but our all slowly perhaps out for you</t>
+  </si>
+  <si>
+    <t>immediately nothing quickly only immediately had finally our suddenly everyone someone let had said gradually normally than your usually than new how have fully them which see how being some have put actually been than exactly let some him its and have let something use primarily there always but only anything say therefore when primarily another partly exactly originally there partly its really your entirely immediately that normally another something their have who particularly recently said them her new already into recently these therefore already someone the basically finally has its not completely totally are all would boy completely during</t>
+  </si>
+  <si>
+    <t>each usually definitely nothing although out sometimes usually although gradually would she has finally put actually the new primarily primarily can basically when would has therefore someone quickly another eventually entirely especially everything recently the than through which entirely get only out usually without has someone everyone actually was exactly really has then when eventually have our old him fully many will therefore was let quickly before definitely new put mainly when into something old put about basically more for but many many totally many after some should after immediately sometimes put originally another its sometimes more see man was</t>
+  </si>
+  <si>
+    <t>everyone your especially our day exactly could use said finally however something from especially generally another during because through while that said which can there where had not with originally another definitely generally many their everything our many slowly therefore into more actually say carefully can these old mostly recently you other therefore now something actually another use everyone the originally totally because mostly however say actually new certainly get she man actually absolutely its are with nothing too something then new put have use which did let with perhaps use mostly someone how should exactly more already had nothing</t>
   </si>
   <si>
     <t>Note for row 140</t>
   </si>
   <si>
-    <t>Person 141</t>
-  </si>
-  <si>
-    <t>Person 142</t>
-  </si>
-  <si>
-    <t>Person 143</t>
-  </si>
-  <si>
-    <t>Person 144</t>
-  </si>
-  <si>
-    <t>Person 145</t>
+    <t>finally way which although let put said some really new recently only particularly mainly said had can initially say use mostly obviously primarily into than say than exactly already now really already which totally quickly see generally too nothing anything there say boy however get who slowly too mainly actually use was mainly now all now has how all immediately first another originally between perhaps should her entirely especially quickly before which these while some new mostly out mostly completely day for about has quickly certainly other was anything more each could had when between totally then your although especially</t>
+  </si>
+  <si>
+    <t>recently then normally someone has before old said absolutely actually where already recently should old recently there his there day mainly they its particularly some would more have and use initially primarily have entirely especially therefore but perhaps our should his totally after therefore his suddenly about suddenly has which been his has into too completely certainly someone something first carefully there then already his for exactly this would now she mainly during his when nothing initially exactly only entirely really some entirely eventually apparently our let initially who carefully primarily had during then where for especially fully use for</t>
+  </si>
+  <si>
+    <t>someone initially mainly into they than new than man everyone for who was basically carefully during new man did being could the while during one our these while with first day that carefully but how although each let apparently first through been immediately old absolutely out had had there being our although apparently finally through while their only who are definitely suddenly where totally you could let gradually although mostly certainly apparently use because about more definitely certainly way one mostly slowly old suddenly then through only which some too eventually originally her completely how anything other obviously generally our</t>
+  </si>
+  <si>
+    <t>now has totally way their another let initially before however entirely finally old see this these exactly really use these there everyone perhaps suddenly slowly partly before day before way said have more slowly being will too would sometimes something already many then each after that are between new new man absolutely that totally only out already day our entirely and through from someone some not then old one out definitely day they originally absolutely which into perhaps carefully its old when let carefully the eventually many there which boy however anything partly without these basically particularly partly she particularly</t>
+  </si>
+  <si>
+    <t>way that out finally slowly had should without always her boy will way finally perhaps immediately immediately him too been mainly use them man eventually who man mainly you and originally then now way carefully said nothing already will then how nothing eventually had can from has apparently the really between these their are where say there recently basically after new normally fully when these see now without its eventually something everything some with suddenly between eventually normally had had she exactly too quickly another completely sometimes definitely suddenly fully particularly and initially actually how have some out then being</t>
   </si>
   <si>
     <t>Note for row 145</t>
   </si>
   <si>
-    <t>Person 146</t>
-  </si>
-  <si>
-    <t>Person 147</t>
-  </si>
-  <si>
-    <t>Person 148</t>
-  </si>
-  <si>
-    <t>Person 149</t>
-  </si>
-  <si>
-    <t>Person 150</t>
+    <t>get not more before finally from there everything have into totally really during between day carefully her old being are they say could slowly should each its everything old but get however suddenly can entirely immediately for and get particularly when while have mainly because without that with recently the everyone basically out been with see originally perhaps said one old when mainly usually certainly anything boy absolutely especially another could let finally are anything where usually everyone can than from put use for can many exactly your new everyone certainly recently slowly with without through nothing its fully day</t>
+  </si>
+  <si>
+    <t>their will many see during through everyone for could many get first sometimes was not her suddenly sometimes finally certainly because new there you new get finally not without are mainly boy exactly normally about where however boy have primarily after been exactly each him obviously who said usually for totally how has how between totally first are therefore should day initially let put should mostly now should that there say would quickly not each while fully say into this about she especially during usually are its mostly normally especially then although new man when slowly many into some first</t>
+  </si>
+  <si>
+    <t>although everything recently old usually her have has already generally really where they already our particularly partly than usually from basically definitely use some more anything something can other his how too being would she one entirely however without said eventually after first during you certainly finally basically their first first normally carefully these slowly however each generally with her another apparently normally because finally mostly definitely this obviously between way into someone when our see obviously one man had totally partly eventually with say you partly being which immediately another see then let and she only one finally our</t>
+  </si>
+  <si>
+    <t>who has our our have totally being the boy see see particularly when for immediately therefore really originally because many originally normally for everyone which said which carefully normally into them she said without anything mostly actually everything initially before entirely more generally one only they with all about nothing finally too all actually certainly everyone because immediately their out something only however immediately originally can his all definitely another because finally let see while one immediately who its only but are say being actually sometimes however was then finally something finally first these too into primarily them other sometimes</t>
+  </si>
+  <si>
+    <t>generally absolutely you mostly put have through carefully our they completely their she her who would get without has especially immediately they everyone gradually during said old boy with usually out boy obviously everyone eventually see old him slowly been mainly one with originally before she her completely someone normally than man suddenly mainly had this day now originally let always and can said use generally for said them about her did they perhaps immediately these originally slowly basically the usually who finally initially old she who who out usually him obviously immediately say now you fully him than initially</t>
   </si>
   <si>
     <t>Note for row 150</t>
@@ -1023,7 +1023,7 @@
         <v>8</v>
       </c>
       <c r="E2" s="2">
-        <v>45939.083750590275</v>
+        <v>45143.102791412035</v>
       </c>
       <c r="F2" t="s">
         <v>9</v>
@@ -1043,7 +1043,7 @@
         <v>12</v>
       </c>
       <c r="E3" s="2">
-        <v>45829.5362181713</v>
+        <v>45697.760646967596</v>
       </c>
       <c r="F3" t="s">
         <v>9</v>
@@ -1060,10 +1060,10 @@
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E4" s="2">
-        <v>45921.96363547454</v>
+        <v>45821.44162861111</v>
       </c>
       <c r="F4" t="s">
         <v>9</v>
@@ -1074,16 +1074,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="2">
-        <v>45033.412505995366</v>
+        <v>45057.88314319444</v>
       </c>
       <c r="F5" t="s">
         <v>9</v>
@@ -1094,19 +1094,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E6" s="2">
-        <v>45807.57715287037</v>
+        <v>45122.707466747685</v>
       </c>
       <c r="F6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1114,16 +1114,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E7" s="2">
-        <v>45529.72817240741</v>
+        <v>45193.430932627314</v>
       </c>
       <c r="F7" t="s">
         <v>9</v>
@@ -1134,16 +1134,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E8" s="2">
-        <v>45408.41613724537</v>
+        <v>46009.90825703704</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -1154,16 +1154,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
         <v>22</v>
       </c>
-      <c r="C9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" t="s">
-        <v>17</v>
-      </c>
       <c r="E9" s="2">
-        <v>44944.57901752315</v>
+        <v>45878.77666171297</v>
       </c>
       <c r="F9" t="s">
         <v>9</v>
@@ -1174,16 +1174,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="E10" s="2">
-        <v>45253.5794340162</v>
+        <v>45076.42203559028</v>
       </c>
       <c r="F10" t="s">
         <v>9</v>
@@ -1194,19 +1194,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="D11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E11" s="2">
-        <v>45506.07808561342</v>
+        <v>45138.48773146991</v>
       </c>
       <c r="F11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1214,16 +1214,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E12" s="2">
-        <v>45185.829828773145</v>
+        <v>45679.28192152778</v>
       </c>
       <c r="F12" t="s">
         <v>9</v>
@@ -1234,16 +1234,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E13" s="2">
-        <v>45742.51713359954</v>
+        <v>45144.16939466435</v>
       </c>
       <c r="F13" t="s">
         <v>9</v>
@@ -1254,16 +1254,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C14" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D14" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E14" s="2">
-        <v>45632.12799172454</v>
+        <v>45078.7568859375</v>
       </c>
       <c r="F14" t="s">
         <v>9</v>
@@ -1274,16 +1274,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D15" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E15" s="2">
-        <v>45683.202009988425</v>
+        <v>45696.449137476855</v>
       </c>
       <c r="F15" t="s">
         <v>9</v>
@@ -1297,16 +1297,16 @@
         <v>33</v>
       </c>
       <c r="C16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="2">
+        <v>45744.10516129629</v>
+      </c>
+      <c r="F16" t="s">
         <v>34</v>
-      </c>
-      <c r="D16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E16" s="2">
-        <v>45299.60556225694</v>
-      </c>
-      <c r="F16" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1314,16 +1314,16 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C17" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D17" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E17" s="2">
-        <v>45569.54600606482</v>
+        <v>45151.89314263889</v>
       </c>
       <c r="F17" t="s">
         <v>9</v>
@@ -1334,16 +1334,16 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C18" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D18" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E18" s="2">
-        <v>45648.98475217592</v>
+        <v>45671.01203032407</v>
       </c>
       <c r="F18" t="s">
         <v>9</v>
@@ -1354,16 +1354,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="D19" t="s">
         <v>8</v>
       </c>
       <c r="E19" s="2">
-        <v>45652.482431909724</v>
+        <v>45304.27519170139</v>
       </c>
       <c r="F19" t="s">
         <v>9</v>
@@ -1374,16 +1374,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C20" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D20" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E20" s="2">
-        <v>45672.585999456016</v>
+        <v>45719.76739822917</v>
       </c>
       <c r="F20" t="s">
         <v>9</v>
@@ -1394,19 +1394,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" t="s">
+        <v>21</v>
+      </c>
+      <c r="D21" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="2">
+        <v>44946.65370927083</v>
+      </c>
+      <c r="F21" t="s">
         <v>40</v>
-      </c>
-      <c r="C21" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21" s="2">
-        <v>45200.90845528935</v>
-      </c>
-      <c r="F21" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1414,16 +1414,16 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C22" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D22" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E22" s="2">
-        <v>45569.973434722226</v>
+        <v>45664.791974085645</v>
       </c>
       <c r="F22" t="s">
         <v>9</v>
@@ -1434,16 +1434,16 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C23" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E23" s="2">
-        <v>45078.2014646412</v>
+        <v>45962.12483390047</v>
       </c>
       <c r="F23" t="s">
         <v>9</v>
@@ -1454,16 +1454,16 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C24" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" s="2">
-        <v>45768.75126085649</v>
+        <v>45598.033099548615</v>
       </c>
       <c r="F24" t="s">
         <v>9</v>
@@ -1474,16 +1474,16 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" t="s">
         <v>45</v>
       </c>
-      <c r="C25" t="s">
-        <v>14</v>
-      </c>
       <c r="D25" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E25" s="2">
-        <v>45703.34899111111</v>
+        <v>45478.49549498843</v>
       </c>
       <c r="F25" t="s">
         <v>9</v>
@@ -1497,13 +1497,13 @@
         <v>46</v>
       </c>
       <c r="C26" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D26" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="E26" s="2">
-        <v>45275.87452703704</v>
+        <v>45202.230008391205</v>
       </c>
       <c r="F26" t="s">
         <v>47</v>
@@ -1517,13 +1517,13 @@
         <v>48</v>
       </c>
       <c r="C27" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="D27" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E27" s="2">
-        <v>45917.18606734954</v>
+        <v>45618.37576520833</v>
       </c>
       <c r="F27" t="s">
         <v>9</v>
@@ -1537,13 +1537,13 @@
         <v>49</v>
       </c>
       <c r="C28" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E28" s="2">
-        <v>45853.9583309838</v>
+        <v>45977.138562002314</v>
       </c>
       <c r="F28" t="s">
         <v>9</v>
@@ -1557,13 +1557,13 @@
         <v>50</v>
       </c>
       <c r="C29" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D29" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E29" s="2">
-        <v>45407.663202881944</v>
+        <v>45815.97288748843</v>
       </c>
       <c r="F29" t="s">
         <v>9</v>
@@ -1577,13 +1577,13 @@
         <v>51</v>
       </c>
       <c r="C30" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D30" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E30" s="2">
-        <v>45966.33900108797</v>
+        <v>45660.64593579861</v>
       </c>
       <c r="F30" t="s">
         <v>9</v>
@@ -1597,13 +1597,13 @@
         <v>52</v>
       </c>
       <c r="C31" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D31" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E31" s="2">
-        <v>45796.18942736111</v>
+        <v>45880.354467268524</v>
       </c>
       <c r="F31" t="s">
         <v>53</v>
@@ -1617,13 +1617,13 @@
         <v>54</v>
       </c>
       <c r="C32" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="D32" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="E32" s="2">
-        <v>45122.4601669213</v>
+        <v>45685.21020480324</v>
       </c>
       <c r="F32" t="s">
         <v>9</v>
@@ -1637,13 +1637,13 @@
         <v>55</v>
       </c>
       <c r="C33" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D33" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E33" s="2">
-        <v>45309.21560297454</v>
+        <v>45612.37371875</v>
       </c>
       <c r="F33" t="s">
         <v>9</v>
@@ -1657,13 +1657,13 @@
         <v>56</v>
       </c>
       <c r="C34" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="D34" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E34" s="2">
-        <v>45296.6208025</v>
+        <v>45494.31045087963</v>
       </c>
       <c r="F34" t="s">
         <v>9</v>
@@ -1680,10 +1680,10 @@
         <v>11</v>
       </c>
       <c r="D35" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E35" s="2">
-        <v>45005.716161261575</v>
+        <v>45060.568756608795</v>
       </c>
       <c r="F35" t="s">
         <v>9</v>
@@ -1697,13 +1697,13 @@
         <v>58</v>
       </c>
       <c r="C36" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D36" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E36" s="2">
-        <v>45987.79329706018</v>
+        <v>45661.90853741898</v>
       </c>
       <c r="F36" t="s">
         <v>59</v>
@@ -1717,13 +1717,13 @@
         <v>60</v>
       </c>
       <c r="C37" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D37" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="E37" s="2">
-        <v>45105.44400030092</v>
+        <v>45534.27098417824</v>
       </c>
       <c r="F37" t="s">
         <v>9</v>
@@ -1737,13 +1737,13 @@
         <v>61</v>
       </c>
       <c r="C38" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="D38" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E38" s="2">
-        <v>45580.57925795139</v>
+        <v>45506.75747222222</v>
       </c>
       <c r="F38" t="s">
         <v>9</v>
@@ -1757,13 +1757,13 @@
         <v>62</v>
       </c>
       <c r="C39" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D39" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E39" s="2">
-        <v>45598.92317759259</v>
+        <v>46021.89227866898</v>
       </c>
       <c r="F39" t="s">
         <v>9</v>
@@ -1777,13 +1777,13 @@
         <v>63</v>
       </c>
       <c r="C40" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
       </c>
       <c r="E40" s="2">
-        <v>45853.977445439814</v>
+        <v>45022.056310960645</v>
       </c>
       <c r="F40" t="s">
         <v>9</v>
@@ -1797,13 +1797,13 @@
         <v>64</v>
       </c>
       <c r="C41" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D41" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E41" s="2">
-        <v>45950.02866524305</v>
+        <v>45680.0072115625</v>
       </c>
       <c r="F41" t="s">
         <v>65</v>
@@ -1817,13 +1817,13 @@
         <v>66</v>
       </c>
       <c r="C42" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="D42" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E42" s="2">
-        <v>45447.725218113424</v>
+        <v>45946.32523164352</v>
       </c>
       <c r="F42" t="s">
         <v>9</v>
@@ -1837,13 +1837,13 @@
         <v>67</v>
       </c>
       <c r="C43" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D43" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E43" s="2">
-        <v>45294.393678796296</v>
+        <v>45973.52818863426</v>
       </c>
       <c r="F43" t="s">
         <v>9</v>
@@ -1857,13 +1857,13 @@
         <v>68</v>
       </c>
       <c r="C44" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="D44" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="E44" s="2">
-        <v>45907.77696243055</v>
+        <v>45982.669965497684</v>
       </c>
       <c r="F44" t="s">
         <v>9</v>
@@ -1877,13 +1877,13 @@
         <v>69</v>
       </c>
       <c r="C45" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D45" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E45" s="2">
-        <v>45946.370073240745</v>
+        <v>45207.11188556713</v>
       </c>
       <c r="F45" t="s">
         <v>9</v>
@@ -1900,10 +1900,10 @@
         <v>11</v>
       </c>
       <c r="D46" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E46" s="2">
-        <v>45787.079176342595</v>
+        <v>45291.52353407408</v>
       </c>
       <c r="F46" t="s">
         <v>71</v>
@@ -1917,13 +1917,13 @@
         <v>72</v>
       </c>
       <c r="C47" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D47" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E47" s="2">
-        <v>45499.78260180556</v>
+        <v>45613.24155820602</v>
       </c>
       <c r="F47" t="s">
         <v>9</v>
@@ -1937,13 +1937,13 @@
         <v>73</v>
       </c>
       <c r="C48" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D48" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E48" s="2">
-        <v>45620.68991914352</v>
+        <v>45425.96323892361</v>
       </c>
       <c r="F48" t="s">
         <v>9</v>
@@ -1960,10 +1960,10 @@
         <v>11</v>
       </c>
       <c r="D49" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E49" s="2">
-        <v>45270.473216620376</v>
+        <v>45990.90592821759</v>
       </c>
       <c r="F49" t="s">
         <v>9</v>
@@ -1977,13 +1977,13 @@
         <v>75</v>
       </c>
       <c r="C50" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D50" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E50" s="2">
-        <v>44954.372456400466</v>
+        <v>45049.124113784725</v>
       </c>
       <c r="F50" t="s">
         <v>9</v>
@@ -1997,13 +1997,13 @@
         <v>76</v>
       </c>
       <c r="C51" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="D51" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E51" s="2">
-        <v>44976.946986967596</v>
+        <v>45941.83024940972</v>
       </c>
       <c r="F51" t="s">
         <v>77</v>
@@ -2017,13 +2017,13 @@
         <v>78</v>
       </c>
       <c r="C52" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D52" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E52" s="2">
-        <v>45260.69861204861</v>
+        <v>44983.69295790509</v>
       </c>
       <c r="F52" t="s">
         <v>9</v>
@@ -2040,10 +2040,10 @@
         <v>11</v>
       </c>
       <c r="D53" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E53" s="2">
-        <v>45683.94826337963</v>
+        <v>45135.63467547453</v>
       </c>
       <c r="F53" t="s">
         <v>9</v>
@@ -2057,13 +2057,13 @@
         <v>80</v>
       </c>
       <c r="C54" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D54" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E54" s="2">
-        <v>45480.6386153125</v>
+        <v>45563.86546690972</v>
       </c>
       <c r="F54" t="s">
         <v>9</v>
@@ -2077,13 +2077,13 @@
         <v>81</v>
       </c>
       <c r="C55" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D55" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E55" s="2">
-        <v>45708.50443408565</v>
+        <v>45020.3392925463</v>
       </c>
       <c r="F55" t="s">
         <v>9</v>
@@ -2097,13 +2097,13 @@
         <v>82</v>
       </c>
       <c r="C56" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="D56" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E56" s="2">
-        <v>45096.415314224534</v>
+        <v>45116.560534097225</v>
       </c>
       <c r="F56" t="s">
         <v>83</v>
@@ -2117,13 +2117,13 @@
         <v>84</v>
       </c>
       <c r="C57" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="D57" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E57" s="2">
-        <v>45257.15166732639</v>
+        <v>45715.693400324075</v>
       </c>
       <c r="F57" t="s">
         <v>9</v>
@@ -2137,13 +2137,13 @@
         <v>85</v>
       </c>
       <c r="C58" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D58" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E58" s="2">
-        <v>44970.072751921296</v>
+        <v>45462.207752511575</v>
       </c>
       <c r="F58" t="s">
         <v>9</v>
@@ -2157,13 +2157,13 @@
         <v>86</v>
       </c>
       <c r="C59" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D59" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E59" s="2">
-        <v>44936.56051846065</v>
+        <v>45442.94714199074</v>
       </c>
       <c r="F59" t="s">
         <v>9</v>
@@ -2177,13 +2177,13 @@
         <v>87</v>
       </c>
       <c r="C60" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="D60" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="E60" s="2">
-        <v>45925.30483523148</v>
+        <v>45917.88822875</v>
       </c>
       <c r="F60" t="s">
         <v>9</v>
@@ -2197,13 +2197,13 @@
         <v>88</v>
       </c>
       <c r="C61" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D61" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E61" s="2">
-        <v>45431.825204340275</v>
+        <v>45660.3972925</v>
       </c>
       <c r="F61" t="s">
         <v>89</v>
@@ -2217,13 +2217,13 @@
         <v>90</v>
       </c>
       <c r="C62" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D62" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E62" s="2">
-        <v>45432.584459074074</v>
+        <v>45244.33806231481</v>
       </c>
       <c r="F62" t="s">
         <v>9</v>
@@ -2237,13 +2237,13 @@
         <v>91</v>
       </c>
       <c r="C63" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D63" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E63" s="2">
-        <v>45649.1409677662</v>
+        <v>45293.99625136574</v>
       </c>
       <c r="F63" t="s">
         <v>9</v>
@@ -2257,13 +2257,13 @@
         <v>92</v>
       </c>
       <c r="C64" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D64" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E64" s="2">
-        <v>45120.495342372684</v>
+        <v>45739.185270104164</v>
       </c>
       <c r="F64" t="s">
         <v>9</v>
@@ -2277,13 +2277,13 @@
         <v>93</v>
       </c>
       <c r="C65" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D65" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E65" s="2">
-        <v>45315.787233518524</v>
+        <v>45452.03619690972</v>
       </c>
       <c r="F65" t="s">
         <v>9</v>
@@ -2297,13 +2297,13 @@
         <v>94</v>
       </c>
       <c r="C66" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D66" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E66" s="2">
-        <v>45756.218865</v>
+        <v>45802.069729930554</v>
       </c>
       <c r="F66" t="s">
         <v>95</v>
@@ -2317,13 +2317,13 @@
         <v>96</v>
       </c>
       <c r="C67" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D67" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E67" s="2">
-        <v>45125.04075400463</v>
+        <v>45587.77622542824</v>
       </c>
       <c r="F67" t="s">
         <v>9</v>
@@ -2337,13 +2337,13 @@
         <v>97</v>
       </c>
       <c r="C68" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D68" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E68" s="2">
-        <v>45174.500609675924</v>
+        <v>44976.783875196765</v>
       </c>
       <c r="F68" t="s">
         <v>9</v>
@@ -2357,13 +2357,13 @@
         <v>98</v>
       </c>
       <c r="C69" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="D69" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E69" s="2">
-        <v>45537.97465888889</v>
+        <v>45102.417371620366</v>
       </c>
       <c r="F69" t="s">
         <v>9</v>
@@ -2377,13 +2377,13 @@
         <v>99</v>
       </c>
       <c r="C70" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D70" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E70" s="2">
-        <v>45008.1236084375</v>
+        <v>45816.34622247685</v>
       </c>
       <c r="F70" t="s">
         <v>9</v>
@@ -2397,13 +2397,13 @@
         <v>100</v>
       </c>
       <c r="C71" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D71" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E71" s="2">
-        <v>45577.340428055555</v>
+        <v>45128.61241459491</v>
       </c>
       <c r="F71" t="s">
         <v>101</v>
@@ -2417,13 +2417,13 @@
         <v>102</v>
       </c>
       <c r="C72" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="D72" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E72" s="2">
-        <v>45989.8054927662</v>
+        <v>45362.548487465276</v>
       </c>
       <c r="F72" t="s">
         <v>9</v>
@@ -2437,13 +2437,13 @@
         <v>103</v>
       </c>
       <c r="C73" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D73" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E73" s="2">
-        <v>45620.44676813658</v>
+        <v>45185.82872722222</v>
       </c>
       <c r="F73" t="s">
         <v>9</v>
@@ -2460,10 +2460,10 @@
         <v>7</v>
       </c>
       <c r="D74" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E74" s="2">
-        <v>45434.01956447917</v>
+        <v>45783.604509502315</v>
       </c>
       <c r="F74" t="s">
         <v>9</v>
@@ -2477,13 +2477,13 @@
         <v>105</v>
       </c>
       <c r="C75" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="D75" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E75" s="2">
-        <v>45230.40996358797</v>
+        <v>45679.71418309028</v>
       </c>
       <c r="F75" t="s">
         <v>9</v>
@@ -2497,13 +2497,13 @@
         <v>106</v>
       </c>
       <c r="C76" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="D76" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E76" s="2">
-        <v>44988.18069271991</v>
+        <v>45737.10757591436</v>
       </c>
       <c r="F76" t="s">
         <v>107</v>
@@ -2517,13 +2517,13 @@
         <v>108</v>
       </c>
       <c r="C77" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D77" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E77" s="2">
-        <v>45594.3411287037</v>
+        <v>45531.011194328705</v>
       </c>
       <c r="F77" t="s">
         <v>9</v>
@@ -2537,13 +2537,13 @@
         <v>109</v>
       </c>
       <c r="C78" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D78" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E78" s="2">
-        <v>45884.97167068287</v>
+        <v>45865.47856950232</v>
       </c>
       <c r="F78" t="s">
         <v>9</v>
@@ -2557,13 +2557,13 @@
         <v>110</v>
       </c>
       <c r="C79" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D79" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E79" s="2">
-        <v>45550.55580299768</v>
+        <v>45991.24701575231</v>
       </c>
       <c r="F79" t="s">
         <v>9</v>
@@ -2577,13 +2577,13 @@
         <v>111</v>
       </c>
       <c r="C80" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="D80" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E80" s="2">
-        <v>45645.67921778935</v>
+        <v>45494.81253793981</v>
       </c>
       <c r="F80" t="s">
         <v>9</v>
@@ -2597,13 +2597,13 @@
         <v>112</v>
       </c>
       <c r="C81" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="D81" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E81" s="2">
-        <v>45896.385059409724</v>
+        <v>45018.91857383102</v>
       </c>
       <c r="F81" t="s">
         <v>113</v>
@@ -2617,13 +2617,13 @@
         <v>114</v>
       </c>
       <c r="C82" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D82" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E82" s="2">
-        <v>45599.25219171296</v>
+        <v>45195.333881805556</v>
       </c>
       <c r="F82" t="s">
         <v>9</v>
@@ -2637,13 +2637,13 @@
         <v>115</v>
       </c>
       <c r="C83" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D83" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E83" s="2">
-        <v>45833.8377603125</v>
+        <v>45144.2159972338</v>
       </c>
       <c r="F83" t="s">
         <v>9</v>
@@ -2657,13 +2657,13 @@
         <v>116</v>
       </c>
       <c r="C84" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D84" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E84" s="2">
-        <v>45977.02372386574</v>
+        <v>45541.17612150463</v>
       </c>
       <c r="F84" t="s">
         <v>9</v>
@@ -2677,13 +2677,13 @@
         <v>117</v>
       </c>
       <c r="C85" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D85" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E85" s="2">
-        <v>45469.1178939699</v>
+        <v>45921.00710207176</v>
       </c>
       <c r="F85" t="s">
         <v>9</v>
@@ -2700,10 +2700,10 @@
         <v>7</v>
       </c>
       <c r="D86" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E86" s="2">
-        <v>45049.45702806713</v>
+        <v>45781.68917100695</v>
       </c>
       <c r="F86" t="s">
         <v>119</v>
@@ -2717,13 +2717,13 @@
         <v>120</v>
       </c>
       <c r="C87" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D87" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E87" s="2">
-        <v>45664.00196659722</v>
+        <v>45605.27464834491</v>
       </c>
       <c r="F87" t="s">
         <v>9</v>
@@ -2737,13 +2737,13 @@
         <v>121</v>
       </c>
       <c r="C88" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="D88" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E88" s="2">
-        <v>45537.84134672454</v>
+        <v>45806.6847171875</v>
       </c>
       <c r="F88" t="s">
         <v>9</v>
@@ -2757,13 +2757,13 @@
         <v>122</v>
       </c>
       <c r="C89" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="D89" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E89" s="2">
-        <v>45761.68908195602</v>
+        <v>45038.293456388885</v>
       </c>
       <c r="F89" t="s">
         <v>9</v>
@@ -2777,13 +2777,13 @@
         <v>123</v>
       </c>
       <c r="C90" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="D90" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E90" s="2">
-        <v>45378.36965071759</v>
+        <v>45255.2180877662</v>
       </c>
       <c r="F90" t="s">
         <v>9</v>
@@ -2797,13 +2797,13 @@
         <v>124</v>
       </c>
       <c r="C91" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D91" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E91" s="2">
-        <v>45453.34148153935</v>
+        <v>45627.365948692124</v>
       </c>
       <c r="F91" t="s">
         <v>125</v>
@@ -2817,13 +2817,13 @@
         <v>126</v>
       </c>
       <c r="C92" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="D92" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E92" s="2">
-        <v>45801.89120465278</v>
+        <v>45855.4849374537</v>
       </c>
       <c r="F92" t="s">
         <v>9</v>
@@ -2837,13 +2837,13 @@
         <v>127</v>
       </c>
       <c r="C93" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D93" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E93" s="2">
-        <v>44965.167293125</v>
+        <v>45929.957528252315</v>
       </c>
       <c r="F93" t="s">
         <v>9</v>
@@ -2857,13 +2857,13 @@
         <v>128</v>
       </c>
       <c r="C94" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D94" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E94" s="2">
-        <v>45066.99887041667</v>
+        <v>45031.54272760417</v>
       </c>
       <c r="F94" t="s">
         <v>9</v>
@@ -2877,13 +2877,13 @@
         <v>129</v>
       </c>
       <c r="C95" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="D95" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E95" s="2">
-        <v>45060.12382320601</v>
+        <v>45043.196392962964</v>
       </c>
       <c r="F95" t="s">
         <v>9</v>
@@ -2897,13 +2897,13 @@
         <v>130</v>
       </c>
       <c r="C96" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D96" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E96" s="2">
-        <v>45750.43364966435</v>
+        <v>45204.895870555556</v>
       </c>
       <c r="F96" t="s">
         <v>131</v>
@@ -2917,13 +2917,13 @@
         <v>132</v>
       </c>
       <c r="C97" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="D97" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E97" s="2">
-        <v>44948.199726736115</v>
+        <v>44929.925646620366</v>
       </c>
       <c r="F97" t="s">
         <v>9</v>
@@ -2937,13 +2937,13 @@
         <v>133</v>
       </c>
       <c r="C98" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="D98" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E98" s="2">
-        <v>45925.95130509259</v>
+        <v>45835.8027225</v>
       </c>
       <c r="F98" t="s">
         <v>9</v>
@@ -2957,13 +2957,13 @@
         <v>134</v>
       </c>
       <c r="C99" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D99" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E99" s="2">
-        <v>45376.73413805556</v>
+        <v>45086.501720451386</v>
       </c>
       <c r="F99" t="s">
         <v>9</v>
@@ -2977,13 +2977,13 @@
         <v>135</v>
       </c>
       <c r="C100" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="D100" t="s">
         <v>12</v>
       </c>
       <c r="E100" s="2">
-        <v>45284.32930309028</v>
+        <v>45104.61304674769</v>
       </c>
       <c r="F100" t="s">
         <v>9</v>
@@ -2997,13 +2997,13 @@
         <v>136</v>
       </c>
       <c r="C101" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D101" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E101" s="2">
-        <v>45485.730412743054</v>
+        <v>45295.220789363426</v>
       </c>
       <c r="F101" t="s">
         <v>137</v>
@@ -3017,13 +3017,13 @@
         <v>138</v>
       </c>
       <c r="C102" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D102" t="s">
         <v>12</v>
       </c>
       <c r="E102" s="2">
-        <v>45471.94407869213</v>
+        <v>45659.3377363426</v>
       </c>
       <c r="F102" t="s">
         <v>9</v>
@@ -3037,13 +3037,13 @@
         <v>139</v>
       </c>
       <c r="C103" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D103" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E103" s="2">
-        <v>44984.07630591435</v>
+        <v>45155.052664386574</v>
       </c>
       <c r="F103" t="s">
         <v>9</v>
@@ -3057,13 +3057,13 @@
         <v>140</v>
       </c>
       <c r="C104" t="s">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="D104" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E104" s="2">
-        <v>45693.30002576389</v>
+        <v>45608.08380554398</v>
       </c>
       <c r="F104" t="s">
         <v>9</v>
@@ -3080,10 +3080,10 @@
         <v>7</v>
       </c>
       <c r="D105" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E105" s="2">
-        <v>45647.8305628588</v>
+        <v>46003.01426872685</v>
       </c>
       <c r="F105" t="s">
         <v>9</v>
@@ -3100,10 +3100,10 @@
         <v>7</v>
       </c>
       <c r="D106" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E106" s="2">
-        <v>45234.76553958333</v>
+        <v>45739.81275774306</v>
       </c>
       <c r="F106" t="s">
         <v>143</v>
@@ -3117,13 +3117,13 @@
         <v>144</v>
       </c>
       <c r="C107" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D107" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E107" s="2">
-        <v>45356.90713854167</v>
+        <v>45100.53655638889</v>
       </c>
       <c r="F107" t="s">
         <v>9</v>
@@ -3137,13 +3137,13 @@
         <v>145</v>
       </c>
       <c r="C108" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D108" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E108" s="2">
-        <v>45638.38134782408</v>
+        <v>44933.57071270833</v>
       </c>
       <c r="F108" t="s">
         <v>9</v>
@@ -3157,13 +3157,13 @@
         <v>146</v>
       </c>
       <c r="C109" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="D109" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E109" s="2">
-        <v>45523.46985637731</v>
+        <v>45065.12355366898</v>
       </c>
       <c r="F109" t="s">
         <v>9</v>
@@ -3177,13 +3177,13 @@
         <v>147</v>
       </c>
       <c r="C110" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D110" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="E110" s="2">
-        <v>45098.57215090278</v>
+        <v>45763.93087628472</v>
       </c>
       <c r="F110" t="s">
         <v>9</v>
@@ -3197,13 +3197,13 @@
         <v>148</v>
       </c>
       <c r="C111" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D111" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E111" s="2">
-        <v>45316.38991462963</v>
+        <v>46015.46855576389</v>
       </c>
       <c r="F111" t="s">
         <v>149</v>
@@ -3217,13 +3217,13 @@
         <v>150</v>
       </c>
       <c r="C112" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D112" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E112" s="2">
-        <v>45901.11137894676</v>
+        <v>45471.93298210648</v>
       </c>
       <c r="F112" t="s">
         <v>9</v>
@@ -3237,13 +3237,13 @@
         <v>151</v>
       </c>
       <c r="C113" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D113" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="E113" s="2">
-        <v>45289.725492893514</v>
+        <v>45111.78447400463</v>
       </c>
       <c r="F113" t="s">
         <v>9</v>
@@ -3257,13 +3257,13 @@
         <v>152</v>
       </c>
       <c r="C114" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D114" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E114" s="2">
-        <v>45112.38598709491</v>
+        <v>45558.33870226852</v>
       </c>
       <c r="F114" t="s">
         <v>9</v>
@@ -3277,13 +3277,13 @@
         <v>153</v>
       </c>
       <c r="C115" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D115" t="s">
         <v>12</v>
       </c>
       <c r="E115" s="2">
-        <v>45350.74865983796</v>
+        <v>45242.59115586805</v>
       </c>
       <c r="F115" t="s">
         <v>9</v>
@@ -3297,13 +3297,13 @@
         <v>154</v>
       </c>
       <c r="C116" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="D116" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E116" s="2">
-        <v>44960.11539047454</v>
+        <v>45968.935523125</v>
       </c>
       <c r="F116" t="s">
         <v>155</v>
@@ -3320,10 +3320,10 @@
         <v>14</v>
       </c>
       <c r="D117" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E117" s="2">
-        <v>45083.66727605324</v>
+        <v>44975.541631875</v>
       </c>
       <c r="F117" t="s">
         <v>9</v>
@@ -3337,13 +3337,13 @@
         <v>157</v>
       </c>
       <c r="C118" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D118" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E118" s="2">
-        <v>45153.225753113424</v>
+        <v>45477.8994446875</v>
       </c>
       <c r="F118" t="s">
         <v>9</v>
@@ -3357,13 +3357,13 @@
         <v>158</v>
       </c>
       <c r="C119" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D119" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E119" s="2">
-        <v>45571.16368668982</v>
+        <v>45791.11059719908</v>
       </c>
       <c r="F119" t="s">
         <v>9</v>
@@ -3377,13 +3377,13 @@
         <v>159</v>
       </c>
       <c r="C120" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D120" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E120" s="2">
-        <v>45324.40736833333</v>
+        <v>45197.949214004635</v>
       </c>
       <c r="F120" t="s">
         <v>9</v>
@@ -3397,13 +3397,13 @@
         <v>160</v>
       </c>
       <c r="C121" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D121" t="s">
         <v>12</v>
       </c>
       <c r="E121" s="2">
-        <v>45152.86527895833</v>
+        <v>45946.68050296296</v>
       </c>
       <c r="F121" t="s">
         <v>161</v>
@@ -3417,13 +3417,13 @@
         <v>162</v>
       </c>
       <c r="C122" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D122" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E122" s="2">
-        <v>45369.06387704861</v>
+        <v>45169.05375190973</v>
       </c>
       <c r="F122" t="s">
         <v>9</v>
@@ -3437,13 +3437,13 @@
         <v>163</v>
       </c>
       <c r="C123" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D123" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E123" s="2">
-        <v>45952.73937552083</v>
+        <v>45313.756019328706</v>
       </c>
       <c r="F123" t="s">
         <v>9</v>
@@ -3457,13 +3457,13 @@
         <v>164</v>
       </c>
       <c r="C124" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D124" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E124" s="2">
-        <v>45768.15889295139</v>
+        <v>45202.72132285879</v>
       </c>
       <c r="F124" t="s">
         <v>9</v>
@@ -3477,13 +3477,13 @@
         <v>165</v>
       </c>
       <c r="C125" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D125" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E125" s="2">
-        <v>45328.20966049768</v>
+        <v>45460.47408533565</v>
       </c>
       <c r="F125" t="s">
         <v>9</v>
@@ -3497,13 +3497,13 @@
         <v>166</v>
       </c>
       <c r="C126" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D126" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E126" s="2">
-        <v>45941.83322111111</v>
+        <v>45105.3390234375</v>
       </c>
       <c r="F126" t="s">
         <v>167</v>
@@ -3517,13 +3517,13 @@
         <v>168</v>
       </c>
       <c r="C127" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D127" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E127" s="2">
-        <v>44933.60669211806</v>
+        <v>45279.23010043982</v>
       </c>
       <c r="F127" t="s">
         <v>9</v>
@@ -3537,13 +3537,13 @@
         <v>169</v>
       </c>
       <c r="C128" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D128" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="E128" s="2">
-        <v>45636.53265616898</v>
+        <v>45082.08718877315</v>
       </c>
       <c r="F128" t="s">
         <v>9</v>
@@ -3557,13 +3557,13 @@
         <v>170</v>
       </c>
       <c r="C129" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D129" t="s">
         <v>8</v>
       </c>
       <c r="E129" s="2">
-        <v>45080.97970648148</v>
+        <v>45062.358714918984</v>
       </c>
       <c r="F129" t="s">
         <v>9</v>
@@ -3577,13 +3577,13 @@
         <v>171</v>
       </c>
       <c r="C130" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="D130" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="E130" s="2">
-        <v>45434.88221524305</v>
+        <v>45905.68349335648</v>
       </c>
       <c r="F130" t="s">
         <v>9</v>
@@ -3597,13 +3597,13 @@
         <v>172</v>
       </c>
       <c r="C131" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D131" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E131" s="2">
-        <v>45239.478362696755</v>
+        <v>45205.43582445601</v>
       </c>
       <c r="F131" t="s">
         <v>173</v>
@@ -3617,13 +3617,13 @@
         <v>174</v>
       </c>
       <c r="C132" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="D132" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E132" s="2">
-        <v>45609.7977209838</v>
+        <v>45490.407541203705</v>
       </c>
       <c r="F132" t="s">
         <v>9</v>
@@ -3637,13 +3637,13 @@
         <v>175</v>
       </c>
       <c r="C133" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D133" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E133" s="2">
-        <v>45504.02472811342</v>
+        <v>45915.94741604167</v>
       </c>
       <c r="F133" t="s">
         <v>9</v>
@@ -3657,13 +3657,13 @@
         <v>176</v>
       </c>
       <c r="C134" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D134" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E134" s="2">
-        <v>45034.250620844905</v>
+        <v>45147.367361655095</v>
       </c>
       <c r="F134" t="s">
         <v>9</v>
@@ -3677,13 +3677,13 @@
         <v>177</v>
       </c>
       <c r="C135" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="D135" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E135" s="2">
-        <v>45122.9723112037</v>
+        <v>45371.36429104167</v>
       </c>
       <c r="F135" t="s">
         <v>9</v>
@@ -3697,13 +3697,13 @@
         <v>178</v>
       </c>
       <c r="C136" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D136" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E136" s="2">
-        <v>45864.103865439814</v>
+        <v>45702.90671173611</v>
       </c>
       <c r="F136" t="s">
         <v>179</v>
@@ -3720,10 +3720,10 @@
         <v>11</v>
       </c>
       <c r="D137" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E137" s="2">
-        <v>45859.88566851852</v>
+        <v>44951.40575826389</v>
       </c>
       <c r="F137" t="s">
         <v>9</v>
@@ -3737,13 +3737,13 @@
         <v>181</v>
       </c>
       <c r="C138" t="s">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="D138" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="E138" s="2">
-        <v>45058.685967337966</v>
+        <v>45708.804541875</v>
       </c>
       <c r="F138" t="s">
         <v>9</v>
@@ -3757,13 +3757,13 @@
         <v>182</v>
       </c>
       <c r="C139" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D139" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E139" s="2">
-        <v>45059.01743425926</v>
+        <v>45718.64279629629</v>
       </c>
       <c r="F139" t="s">
         <v>9</v>
@@ -3777,13 +3777,13 @@
         <v>183</v>
       </c>
       <c r="C140" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D140" t="s">
         <v>8</v>
       </c>
       <c r="E140" s="2">
-        <v>45954.66003320602</v>
+        <v>45117.51364377315</v>
       </c>
       <c r="F140" t="s">
         <v>9</v>
@@ -3797,13 +3797,13 @@
         <v>184</v>
       </c>
       <c r="C141" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D141" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E141" s="2">
-        <v>45834.46553559028</v>
+        <v>45866.755907280094</v>
       </c>
       <c r="F141" t="s">
         <v>185</v>
@@ -3817,13 +3817,13 @@
         <v>186</v>
       </c>
       <c r="C142" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="D142" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="E142" s="2">
-        <v>45459.17694643518</v>
+        <v>45303.916257268516</v>
       </c>
       <c r="F142" t="s">
         <v>9</v>
@@ -3837,13 +3837,13 @@
         <v>187</v>
       </c>
       <c r="C143" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="D143" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E143" s="2">
-        <v>45640.99325179398</v>
+        <v>45383.74967056713</v>
       </c>
       <c r="F143" t="s">
         <v>9</v>
@@ -3857,13 +3857,13 @@
         <v>188</v>
       </c>
       <c r="C144" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D144" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E144" s="2">
-        <v>45915.05035445602</v>
+        <v>45396.83874436343</v>
       </c>
       <c r="F144" t="s">
         <v>9</v>
@@ -3877,13 +3877,13 @@
         <v>189</v>
       </c>
       <c r="C145" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="D145" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E145" s="2">
-        <v>45366.18571457176</v>
+        <v>45323.514683587964</v>
       </c>
       <c r="F145" t="s">
         <v>9</v>
@@ -3897,13 +3897,13 @@
         <v>190</v>
       </c>
       <c r="C146" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D146" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E146" s="2">
-        <v>45407.01464355324</v>
+        <v>45869.27488871528</v>
       </c>
       <c r="F146" t="s">
         <v>191</v>
@@ -3917,13 +3917,13 @@
         <v>192</v>
       </c>
       <c r="C147" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D147" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E147" s="2">
-        <v>45363.96879295139</v>
+        <v>45442.23598269676</v>
       </c>
       <c r="F147" t="s">
         <v>9</v>
@@ -3937,13 +3937,13 @@
         <v>193</v>
       </c>
       <c r="C148" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="D148" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E148" s="2">
-        <v>44995.362212685184</v>
+        <v>45220.314411099534</v>
       </c>
       <c r="F148" t="s">
         <v>9</v>
@@ -3957,13 +3957,13 @@
         <v>194</v>
       </c>
       <c r="C149" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D149" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E149" s="2">
-        <v>45588.39076627315</v>
+        <v>45600.72355949074</v>
       </c>
       <c r="F149" t="s">
         <v>9</v>
@@ -3977,13 +3977,13 @@
         <v>195</v>
       </c>
       <c r="C150" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="D150" t="s">
         <v>8</v>
       </c>
       <c r="E150" s="2">
-        <v>45484.44575236111</v>
+        <v>45128.62223987268</v>
       </c>
       <c r="F150" t="s">
         <v>9</v>
@@ -3997,13 +3997,13 @@
         <v>196</v>
       </c>
       <c r="C151" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D151" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E151" s="2">
-        <v>44956.94424225694</v>
+        <v>45042.47163914352</v>
       </c>
       <c r="F151" t="s">
         <v>197</v>

</xml_diff>